<commit_message>
End documentation of Parameter_unc_nonlin.ipynb
Propagated COV_IS computed from DE with MC!! Plots to be saved but dynamic results saved
</commit_message>
<xml_diff>
--- a/Parameter_estimation/uit_real_R2+batch_april24_FIM_COV_sigma_01-12-2025.xlsx
+++ b/Parameter_estimation/uit_real_R2+batch_april24_FIM_COV_sigma_01-12-2025.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10530006_polimi_it/Documents/Work_cloud/DOTTORATO/Modelling/Pilot_plant/Parameter_estimation/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_ED70979F7DD2020A4F50F93CA6B0D01A6D9808E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01D1213C-6F0F-48E6-9675-E4EB344A8D05}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FIM" sheetId="1" r:id="rId1"/>
@@ -12,7 +18,7 @@
     <sheet name="Parameter_Std_Dev" sheetId="3" r:id="rId3"/>
     <sheet name="Parameter_Significance" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -76,8 +82,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -129,24 +135,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -184,7 +199,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -218,6 +233,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -252,9 +268,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -427,11 +444,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -475,33 +492,33 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>41721207236.31335</v>
+        <v>41721207236.313347</v>
       </c>
       <c r="C2">
-        <v>3493080.126443158</v>
+        <v>3493080.1264431579</v>
       </c>
       <c r="D2">
-        <v>34549075388.48124</v>
+        <v>34549075388.481239</v>
       </c>
       <c r="E2">
         <v>109684106.4474176</v>
       </c>
       <c r="F2">
-        <v>-473890193.0938991</v>
+        <v>-473890193.09389907</v>
       </c>
       <c r="G2">
-        <v>76297121892.75858</v>
+        <v>76297121892.758575</v>
       </c>
       <c r="H2">
-        <v>699544.907987964</v>
+        <v>699544.90798796399</v>
       </c>
       <c r="I2">
-        <v>-2325588.429415844</v>
+        <v>-2325588.4294158439</v>
       </c>
       <c r="J2">
         <v>135.6478942481034</v>
@@ -510,113 +527,113 @@
         <v>-2359621312976.292</v>
       </c>
       <c r="L2">
-        <v>402336557.0347567</v>
+        <v>402336557.03475672</v>
       </c>
       <c r="M2">
-        <v>-750708030461507.8</v>
+        <v>-750708030461507.75</v>
       </c>
       <c r="N2">
         <v>4631802344998073</v>
       </c>
       <c r="O2">
-        <v>-79438170.22581354</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15">
+        <v>-79438170.225813538</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>3493080.126443158</v>
+        <v>3493080.1264431579</v>
       </c>
       <c r="C3">
-        <v>292.4582756172771</v>
+        <v>292.45827561727708</v>
       </c>
       <c r="D3">
-        <v>2892598.195609274</v>
+        <v>2892598.1956092739</v>
       </c>
       <c r="E3">
         <v>9233.603082187803</v>
       </c>
       <c r="F3">
-        <v>-39732.16555359533</v>
+        <v>-39732.165553595332</v>
       </c>
       <c r="G3">
-        <v>6456339.200161286</v>
+        <v>6456339.2001612857</v>
       </c>
       <c r="H3">
-        <v>69.98249276779286</v>
+        <v>69.982492767792863</v>
       </c>
       <c r="I3">
-        <v>-194.6534422659456</v>
+        <v>-194.65344226594561</v>
       </c>
       <c r="J3">
-        <v>-4.898931486693635</v>
+        <v>-4.8989314866936349</v>
       </c>
       <c r="K3">
-        <v>-197557710.1371082</v>
+        <v>-197557710.13710821</v>
       </c>
       <c r="L3">
-        <v>33685.36161055136</v>
+        <v>33685.361610551357</v>
       </c>
       <c r="M3">
-        <v>-62852531697.98212</v>
+        <v>-62852531697.982117</v>
       </c>
       <c r="N3">
-        <v>387794580488.6255</v>
+        <v>387794580488.62549</v>
       </c>
       <c r="O3">
-        <v>-6696.467379527558</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15">
+        <v>-6696.4673795275576</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>34549075388.48124</v>
+        <v>34549075388.481239</v>
       </c>
       <c r="C4">
-        <v>2892598.195609274</v>
+        <v>2892598.1956092739</v>
       </c>
       <c r="D4">
         <v>28609878188.30407</v>
       </c>
       <c r="E4">
-        <v>90828594.16121636</v>
+        <v>90828594.161216363</v>
       </c>
       <c r="F4">
-        <v>-392425987.9759104</v>
+        <v>-392425987.97591043</v>
       </c>
       <c r="G4">
-        <v>63180953895.48826</v>
+        <v>63180953895.488258</v>
       </c>
       <c r="H4">
-        <v>579233.8292684453</v>
+        <v>579233.82926844526</v>
       </c>
       <c r="I4">
-        <v>-1924911.567724489</v>
+        <v>-1924911.5677244889</v>
       </c>
       <c r="J4">
-        <v>1007.385618622653</v>
+        <v>1007.3856186226531</v>
       </c>
       <c r="K4">
-        <v>-1953987924483.727</v>
+        <v>-1953987924483.7271</v>
       </c>
       <c r="L4">
-        <v>333172488.5193721</v>
+        <v>333172488.51937211</v>
       </c>
       <c r="M4">
-        <v>-621656812714365.4</v>
+        <v>-621656812714365.38</v>
       </c>
       <c r="N4">
         <v>3835567713062442</v>
       </c>
       <c r="O4">
-        <v>-65782311.9621631</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15">
+        <v>-65782311.962163098</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -627,19 +644,19 @@
         <v>9233.603082187803</v>
       </c>
       <c r="D5">
-        <v>90828594.16121636</v>
+        <v>90828594.161216363</v>
       </c>
       <c r="E5">
-        <v>1472104.268985489</v>
+        <v>1472104.2689854889</v>
       </c>
       <c r="F5">
-        <v>-2575781.181908947</v>
+        <v>-2575781.1819089469</v>
       </c>
       <c r="G5">
         <v>1809313062.638026</v>
       </c>
       <c r="H5">
-        <v>269361.2489534735</v>
+        <v>269361.24895347352</v>
       </c>
       <c r="I5">
         <v>-5983.913224349104</v>
@@ -648,80 +665,80 @@
         <v>-116378.5110605714</v>
       </c>
       <c r="K5">
-        <v>-6203372990.374132</v>
+        <v>-6203372990.3741322</v>
       </c>
       <c r="L5">
         <v>1057746.280846549</v>
       </c>
       <c r="M5">
-        <v>-1973591735056.972</v>
+        <v>-1973591735056.9719</v>
       </c>
       <c r="N5">
         <v>12176949940661.93</v>
       </c>
       <c r="O5">
-        <v>-1275313.626844772</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15">
+        <v>-1275313.6268447719</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B6">
-        <v>-473890193.0938991</v>
+        <v>-473890193.09389907</v>
       </c>
       <c r="C6">
-        <v>-39732.16555359533</v>
+        <v>-39732.165553595332</v>
       </c>
       <c r="D6">
-        <v>-392425987.9759104</v>
+        <v>-392425987.97591043</v>
       </c>
       <c r="E6">
-        <v>-2575781.181908947</v>
+        <v>-2575781.1819089469</v>
       </c>
       <c r="F6">
-        <v>6953347.978476102</v>
+        <v>6953347.9784761025</v>
       </c>
       <c r="G6">
         <v>-2677254971.609931</v>
       </c>
       <c r="H6">
-        <v>-304922.9910737784</v>
+        <v>-304922.99107377842</v>
       </c>
       <c r="I6">
         <v>25733.42390021863</v>
       </c>
       <c r="J6">
-        <v>110348.1400979854</v>
+        <v>110348.14009798539</v>
       </c>
       <c r="K6">
         <v>26801729608.2603</v>
       </c>
       <c r="L6">
-        <v>-4569987.352516211</v>
+        <v>-4569987.3525162106</v>
       </c>
       <c r="M6">
-        <v>8526981373949.264</v>
+        <v>8526981373949.2637</v>
       </c>
       <c r="N6">
-        <v>-52610754075114.67</v>
+        <v>-52610754075114.672</v>
       </c>
       <c r="O6">
-        <v>2088542.54518911</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15">
+        <v>2088542.5451891101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B7">
-        <v>76297121892.75858</v>
+        <v>76297121892.758575</v>
       </c>
       <c r="C7">
-        <v>6456339.200161287</v>
+        <v>6456339.2001612866</v>
       </c>
       <c r="D7">
-        <v>63180953895.48826</v>
+        <v>63180953895.488258</v>
       </c>
       <c r="E7">
         <v>1809313062.638026</v>
@@ -730,22 +747,22 @@
         <v>-2677254971.609931</v>
       </c>
       <c r="G7">
-        <v>2325994330108.809</v>
+        <v>2325994330108.8091</v>
       </c>
       <c r="H7">
-        <v>364694421.1564111</v>
+        <v>364694421.15641111</v>
       </c>
       <c r="I7">
-        <v>-4101154.795255713</v>
+        <v>-4101154.7952557132</v>
       </c>
       <c r="J7">
-        <v>-157698594.5607708</v>
+        <v>-157698594.56077081</v>
       </c>
       <c r="K7">
-        <v>-4315102561936.339</v>
+        <v>-4315102561936.3389</v>
       </c>
       <c r="L7">
-        <v>735783060.078647</v>
+        <v>735783060.07864702</v>
       </c>
       <c r="M7">
         <v>-1372840925738698</v>
@@ -757,65 +774,65 @@
         <v>-1593910278.227237</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B8">
-        <v>699544.907987964</v>
+        <v>699544.90798796399</v>
       </c>
       <c r="C8">
-        <v>69.98249276779286</v>
+        <v>69.982492767792863</v>
       </c>
       <c r="D8">
-        <v>579233.8292684453</v>
+        <v>579233.82926844526</v>
       </c>
       <c r="E8">
-        <v>269361.2489534735</v>
+        <v>269361.24895347352</v>
       </c>
       <c r="F8">
-        <v>-304922.9910737784</v>
+        <v>-304922.99107377842</v>
       </c>
       <c r="G8">
-        <v>364694421.1564111</v>
+        <v>364694421.15641111</v>
       </c>
       <c r="H8">
-        <v>60641.73419830743</v>
+        <v>60641.734198307429</v>
       </c>
       <c r="I8">
-        <v>-29.59967882334836</v>
+        <v>-29.599678823348359</v>
       </c>
       <c r="J8">
-        <v>-27213.25007100976</v>
+        <v>-27213.250071009759</v>
       </c>
       <c r="K8">
-        <v>-39560026.10664106</v>
+        <v>-39560026.106641062</v>
       </c>
       <c r="L8">
-        <v>6747.544831988003</v>
+        <v>6747.5448319880034</v>
       </c>
       <c r="M8">
         <v>-12583903663.96908</v>
       </c>
       <c r="N8">
-        <v>77657865526.52231</v>
+        <v>77657865526.522308</v>
       </c>
       <c r="O8">
-        <v>-242910.1535498238</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15">
+        <v>-242910.15354982379</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9">
-        <v>-2325588.429415844</v>
+        <v>-2325588.4294158439</v>
       </c>
       <c r="C9">
-        <v>-194.6534422659456</v>
+        <v>-194.65344226594561</v>
       </c>
       <c r="D9">
-        <v>-1924911.567724489</v>
+        <v>-1924911.5677244889</v>
       </c>
       <c r="E9">
         <v>-5983.913224349104</v>
@@ -824,16 +841,16 @@
         <v>25733.42390021863</v>
       </c>
       <c r="G9">
-        <v>-4101154.795255713</v>
+        <v>-4101154.7952557132</v>
       </c>
       <c r="H9">
-        <v>-29.59967882334835</v>
+        <v>-29.599678823348349</v>
       </c>
       <c r="I9">
-        <v>965.0177995561454</v>
+        <v>965.01779955614541</v>
       </c>
       <c r="J9">
-        <v>848.5708878561088</v>
+        <v>848.57088785610881</v>
       </c>
       <c r="K9">
         <v>131526117.8309859</v>
@@ -842,16 +859,16 @@
         <v>-22375.83598448581</v>
       </c>
       <c r="M9">
-        <v>41752650917.45715</v>
+        <v>41752650917.457153</v>
       </c>
       <c r="N9">
-        <v>-257609934187.7426</v>
+        <v>-257609934187.74261</v>
       </c>
       <c r="O9">
-        <v>4164.221326678357</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15">
+        <v>4164.2213266783574</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -859,22 +876,22 @@
         <v>135.6478942481034</v>
       </c>
       <c r="C10">
-        <v>-4.898931486693636</v>
+        <v>-4.8989314866936358</v>
       </c>
       <c r="D10">
-        <v>1007.385618622653</v>
+        <v>1007.3856186226531</v>
       </c>
       <c r="E10">
         <v>-116378.5110605715</v>
       </c>
       <c r="F10">
-        <v>110348.1400979854</v>
+        <v>110348.14009798539</v>
       </c>
       <c r="G10">
-        <v>-157698594.5607708</v>
+        <v>-157698594.56077081</v>
       </c>
       <c r="H10">
-        <v>-27213.25007100976</v>
+        <v>-27213.250071009759</v>
       </c>
       <c r="I10">
         <v>848.5708878561087</v>
@@ -886,19 +903,19 @@
         <v>-4135.448299562292</v>
       </c>
       <c r="L10">
-        <v>55.6350907785755</v>
+        <v>55.635090778575503</v>
       </c>
       <c r="M10">
         <v>-106514360.9282804</v>
       </c>
       <c r="N10">
-        <v>618226858.041615</v>
+        <v>618226858.04161501</v>
       </c>
       <c r="O10">
-        <v>105944.6957167672</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15">
+        <v>105944.69571676719</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -906,22 +923,22 @@
         <v>-2359621312976.292</v>
       </c>
       <c r="C11">
-        <v>-197557710.1371082</v>
+        <v>-197557710.13710821</v>
       </c>
       <c r="D11">
-        <v>-1953987924483.727</v>
+        <v>-1953987924483.7271</v>
       </c>
       <c r="E11">
-        <v>-6203372990.374133</v>
+        <v>-6203372990.3741331</v>
       </c>
       <c r="F11">
         <v>26801729608.2603</v>
       </c>
       <c r="G11">
-        <v>-4315102561936.339</v>
+        <v>-4315102561936.3389</v>
       </c>
       <c r="H11">
-        <v>-39560026.10664105</v>
+        <v>-39560026.106641047</v>
       </c>
       <c r="I11">
         <v>131526117.8309859</v>
@@ -933,83 +950,83 @@
         <v>133452820228690.2</v>
       </c>
       <c r="L11">
-        <v>-22754900629.5556</v>
+        <v>-22754900629.555599</v>
       </c>
       <c r="M11">
-        <v>4.245770446302703E+16</v>
+        <v>4.2457704463027032E+16</v>
       </c>
       <c r="N11">
-        <v>-2.619602923780852E+17</v>
+        <v>-2.6196029237808518E+17</v>
       </c>
       <c r="O11">
-        <v>4492759863.625604</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15">
+        <v>4492759863.6256037</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B12">
-        <v>402336557.0347567</v>
+        <v>402336557.03475672</v>
       </c>
       <c r="C12">
-        <v>33685.36161055136</v>
+        <v>33685.361610551357</v>
       </c>
       <c r="D12">
-        <v>333172488.5193721</v>
+        <v>333172488.51937211</v>
       </c>
       <c r="E12">
         <v>1057746.280846549</v>
       </c>
       <c r="F12">
-        <v>-4569987.352516211</v>
+        <v>-4569987.3525162106</v>
       </c>
       <c r="G12">
-        <v>735783060.078647</v>
+        <v>735783060.07864702</v>
       </c>
       <c r="H12">
-        <v>6747.544831988002</v>
+        <v>6747.5448319880024</v>
       </c>
       <c r="I12">
         <v>-22375.83598448581</v>
       </c>
       <c r="J12">
-        <v>55.6350907785755</v>
+        <v>55.635090778575503</v>
       </c>
       <c r="K12">
-        <v>-22754900629.5556</v>
+        <v>-22754900629.555599</v>
       </c>
       <c r="L12">
-        <v>3879917.4745141</v>
+        <v>3879917.4745140998</v>
       </c>
       <c r="M12">
-        <v>-7239424538496.902</v>
+        <v>-7239424538496.9023</v>
       </c>
       <c r="N12">
-        <v>44666610930788.69</v>
+        <v>44666610930788.688</v>
       </c>
       <c r="O12">
         <v>-766080.2506618374</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B13">
-        <v>-750708030461507.8</v>
+        <v>-750708030461507.75</v>
       </c>
       <c r="C13">
-        <v>-62852531697.98212</v>
+        <v>-62852531697.982117</v>
       </c>
       <c r="D13">
-        <v>-621656812714365.4</v>
+        <v>-621656812714365.38</v>
       </c>
       <c r="E13">
-        <v>-1973591735056.972</v>
+        <v>-1973591735056.9719</v>
       </c>
       <c r="F13">
-        <v>8526981373949.265</v>
+        <v>8526981373949.2646</v>
       </c>
       <c r="G13">
         <v>-1372840925738698</v>
@@ -1018,28 +1035,28 @@
         <v>-12583903663.96908</v>
       </c>
       <c r="I13">
-        <v>41752650917.45715</v>
+        <v>41752650917.457153</v>
       </c>
       <c r="J13">
         <v>-106514360.9282804</v>
       </c>
       <c r="K13">
-        <v>4.245770446302703E+16</v>
+        <v>4.2457704463027032E+16</v>
       </c>
       <c r="L13">
-        <v>-7239424538496.902</v>
+        <v>-7239424538496.9023</v>
       </c>
       <c r="M13">
-        <v>1.350783054607149E+19</v>
+        <v>1.3507830546071491E+19</v>
       </c>
       <c r="N13">
         <v>-8.33421232053171E+19</v>
       </c>
       <c r="O13">
-        <v>1429381826137.443</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15">
+        <v>1429381826137.4431</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -1047,7 +1064,7 @@
         <v>4631802344998073</v>
       </c>
       <c r="C14">
-        <v>387794580488.6255</v>
+        <v>387794580488.62549</v>
       </c>
       <c r="D14">
         <v>3835567713062442</v>
@@ -1056,81 +1073,81 @@
         <v>12176949940661.93</v>
       </c>
       <c r="F14">
-        <v>-52610754075114.67</v>
+        <v>-52610754075114.672</v>
       </c>
       <c r="G14">
         <v>8470393066992937</v>
       </c>
       <c r="H14">
-        <v>77657865526.52231</v>
+        <v>77657865526.522308</v>
       </c>
       <c r="I14">
-        <v>-257609934187.7426</v>
+        <v>-257609934187.74261</v>
       </c>
       <c r="J14">
-        <v>618226858.041615</v>
+        <v>618226858.04161501</v>
       </c>
       <c r="K14">
-        <v>-2.619602923780852E+17</v>
+        <v>-2.6196029237808518E+17</v>
       </c>
       <c r="L14">
-        <v>44666610930788.69</v>
+        <v>44666610930788.688</v>
       </c>
       <c r="M14">
         <v>-8.33421232053171E+19</v>
       </c>
       <c r="N14">
-        <v>5.142135512306901E+20</v>
+        <v>5.1421355123069013E+20</v>
       </c>
       <c r="O14">
-        <v>-8819214715465.303</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15">
+        <v>-8819214715465.3027</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B15">
-        <v>-79438170.22581354</v>
+        <v>-79438170.225813538</v>
       </c>
       <c r="C15">
-        <v>-6696.467379527558</v>
+        <v>-6696.4673795275576</v>
       </c>
       <c r="D15">
-        <v>-65782311.9621631</v>
+        <v>-65782311.962163098</v>
       </c>
       <c r="E15">
-        <v>-1275313.626844772</v>
+        <v>-1275313.6268447719</v>
       </c>
       <c r="F15">
-        <v>2088542.54518911</v>
+        <v>2088542.5451891101</v>
       </c>
       <c r="G15">
-        <v>-1593910278.227238</v>
+        <v>-1593910278.2272379</v>
       </c>
       <c r="H15">
-        <v>-242910.1535498238</v>
+        <v>-242910.15354982379</v>
       </c>
       <c r="I15">
-        <v>4164.221326678358</v>
+        <v>4164.2213266783583</v>
       </c>
       <c r="J15">
-        <v>105944.6957167672</v>
+        <v>105944.69571676719</v>
       </c>
       <c r="K15">
-        <v>4492759863.625604</v>
+        <v>4492759863.6256037</v>
       </c>
       <c r="L15">
         <v>-766080.2506618374</v>
       </c>
       <c r="M15">
-        <v>1429381826137.443</v>
+        <v>1429381826137.4431</v>
       </c>
       <c r="N15">
-        <v>-8819214715465.303</v>
+        <v>-8819214715465.3027</v>
       </c>
       <c r="O15">
-        <v>1114980.287219437</v>
+        <v>1114980.2872194371</v>
       </c>
     </row>
   </sheetData>
@@ -1139,11 +1156,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1187,662 +1204,662 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
-        <v>0.005518803211410026</v>
-      </c>
-      <c r="C2">
+      <c r="B2" s="2">
+        <v>5.5188032114100258E-3</v>
+      </c>
+      <c r="C2" s="2">
         <v>-1.281185083261752</v>
       </c>
-      <c r="D2">
-        <v>0.009380799395582801</v>
-      </c>
-      <c r="E2">
-        <v>0.01095790147515066</v>
-      </c>
-      <c r="F2">
-        <v>-0.0004272390359116183</v>
-      </c>
-      <c r="G2">
-        <v>-8.312616845254974E-06</v>
-      </c>
-      <c r="H2">
-        <v>0.003066539244928898</v>
-      </c>
-      <c r="I2">
-        <v>-0.004107062867967842</v>
-      </c>
-      <c r="J2">
-        <v>-0.0003301662587709451</v>
-      </c>
-      <c r="K2">
-        <v>0.0002184844601154352</v>
-      </c>
-      <c r="L2">
-        <v>-0.089358106878329</v>
-      </c>
-      <c r="M2">
-        <v>1.818993130703116E-08</v>
-      </c>
-      <c r="N2">
-        <v>3.144345371634074E-09</v>
-      </c>
-      <c r="O2">
-        <v>0.0009022319796738209</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15">
+      <c r="D2" s="2">
+        <v>9.3807993955828013E-3</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1.0957901475150659E-2</v>
+      </c>
+      <c r="F2" s="2">
+        <v>-4.2723903591161829E-4</v>
+      </c>
+      <c r="G2" s="2">
+        <v>-8.3126168452549737E-6</v>
+      </c>
+      <c r="H2" s="2">
+        <v>3.066539244928898E-3</v>
+      </c>
+      <c r="I2" s="2">
+        <v>-4.1070628679678424E-3</v>
+      </c>
+      <c r="J2" s="2">
+        <v>-3.3016625877094511E-4</v>
+      </c>
+      <c r="K2" s="2">
+        <v>2.1848446011543519E-4</v>
+      </c>
+      <c r="L2" s="2">
+        <v>-8.9358106878328999E-2</v>
+      </c>
+      <c r="M2" s="2">
+        <v>1.818993130703116E-8</v>
+      </c>
+      <c r="N2" s="2">
+        <v>3.1443453716340739E-9</v>
+      </c>
+      <c r="O2" s="2">
+        <v>9.0223197967382088E-4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
-        <v>-1.281185253148441</v>
-      </c>
-      <c r="C3">
-        <v>3631.269378144471</v>
-      </c>
-      <c r="D3">
-        <v>3.744851095872072</v>
-      </c>
-      <c r="E3">
+      <c r="B3" s="2">
+        <v>-1.2811852531484409</v>
+      </c>
+      <c r="C3" s="2">
+        <v>3631.2693781444709</v>
+      </c>
+      <c r="D3" s="2">
+        <v>3.7448510958720722</v>
+      </c>
+      <c r="E3" s="2">
         <v>-15.23403571937329</v>
       </c>
-      <c r="F3">
-        <v>0.3213108383819038</v>
-      </c>
-      <c r="G3">
-        <v>0.01077489179536311</v>
-      </c>
-      <c r="H3">
-        <v>-3.46960110608178</v>
-      </c>
-      <c r="I3">
-        <v>-2.01918612809303</v>
-      </c>
-      <c r="J3">
-        <v>0.05866940201676343</v>
-      </c>
-      <c r="K3">
-        <v>0.03054748173963229</v>
-      </c>
-      <c r="L3">
+      <c r="F3" s="2">
+        <v>0.32131083838190377</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1.077489179536311E-2</v>
+      </c>
+      <c r="H3" s="2">
+        <v>-3.4696011060817802</v>
+      </c>
+      <c r="I3" s="2">
+        <v>-2.0191861280930299</v>
+      </c>
+      <c r="J3" s="2">
+        <v>5.8669402016763433E-2</v>
+      </c>
+      <c r="K3" s="2">
+        <v>3.0547481739632291E-2</v>
+      </c>
+      <c r="L3" s="2">
         <v>180.7472294434491</v>
       </c>
-      <c r="M3">
-        <v>0.000128168482600256</v>
-      </c>
-      <c r="N3">
-        <v>1.688887217419972E-06</v>
-      </c>
-      <c r="O3">
+      <c r="M3" s="2">
+        <v>1.2816848260025599E-4</v>
+      </c>
+      <c r="N3" s="2">
+        <v>1.688887217419972E-6</v>
+      </c>
+      <c r="O3" s="2">
         <v>-1.759378776425188</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4">
-        <v>0.009380768605441264</v>
-      </c>
-      <c r="C4">
+      <c r="B4" s="2">
+        <v>9.3807686054412642E-3</v>
+      </c>
+      <c r="C4" s="2">
         <v>3.744855720776008</v>
       </c>
-      <c r="D4">
-        <v>0.9467481985113186</v>
-      </c>
-      <c r="E4">
-        <v>0.01420900907360112</v>
-      </c>
-      <c r="F4">
-        <v>-0.00669080574452878</v>
-      </c>
-      <c r="G4">
-        <v>-3.046241743026999E-05</v>
-      </c>
-      <c r="H4">
-        <v>0.075418954986732</v>
-      </c>
-      <c r="I4">
-        <v>-0.4271095134620501</v>
-      </c>
-      <c r="J4">
-        <v>-0.005926121166513382</v>
-      </c>
-      <c r="K4">
-        <v>0.01244898408240578</v>
-      </c>
-      <c r="L4">
-        <v>-1.585900380645262</v>
-      </c>
-      <c r="M4">
-        <v>3.259381408055921E-06</v>
-      </c>
-      <c r="N4">
-        <v>-1.419645007756101E-07</v>
-      </c>
-      <c r="O4">
-        <v>-0.00207909202861432</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15">
+      <c r="D4" s="2">
+        <v>0.94674819851131864</v>
+      </c>
+      <c r="E4" s="2">
+        <v>1.420900907360112E-2</v>
+      </c>
+      <c r="F4" s="2">
+        <v>-6.69080574452878E-3</v>
+      </c>
+      <c r="G4" s="2">
+        <v>-3.0462417430269991E-5</v>
+      </c>
+      <c r="H4" s="2">
+        <v>7.5418954986731998E-2</v>
+      </c>
+      <c r="I4" s="2">
+        <v>-0.42710951346205012</v>
+      </c>
+      <c r="J4" s="2">
+        <v>-5.9261211665133824E-3</v>
+      </c>
+      <c r="K4" s="2">
+        <v>1.244898408240578E-2</v>
+      </c>
+      <c r="L4" s="2">
+        <v>-1.5859003806452621</v>
+      </c>
+      <c r="M4" s="2">
+        <v>3.2593814080559211E-6</v>
+      </c>
+      <c r="N4" s="2">
+        <v>-1.419645007756101E-7</v>
+      </c>
+      <c r="O4" s="2">
+        <v>-2.0790920286143199E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5">
-        <v>0.01095789896481504</v>
-      </c>
-      <c r="C5">
+      <c r="B5" s="2">
+        <v>1.0957898964815039E-2</v>
+      </c>
+      <c r="C5" s="2">
         <v>-15.23403620821138</v>
       </c>
-      <c r="D5">
-        <v>0.01420886985666749</v>
-      </c>
-      <c r="E5">
-        <v>1.39974201603932</v>
-      </c>
-      <c r="F5">
-        <v>-0.0002147414670007788</v>
-      </c>
-      <c r="G5">
-        <v>-0.0008843680080651921</v>
-      </c>
-      <c r="H5">
+      <c r="D5" s="2">
+        <v>1.4208869856667489E-2</v>
+      </c>
+      <c r="E5" s="2">
+        <v>1.3997420160393199</v>
+      </c>
+      <c r="F5" s="2">
+        <v>-2.147414670007788E-4</v>
+      </c>
+      <c r="G5" s="2">
+        <v>-8.8436800806519214E-4</v>
+      </c>
+      <c r="H5" s="2">
         <v>-0.1180731146586307</v>
       </c>
-      <c r="I5">
-        <v>0.005496009783752896</v>
-      </c>
-      <c r="J5">
-        <v>0.008167329773988641</v>
-      </c>
-      <c r="K5">
-        <v>0.0003447086993209412</v>
-      </c>
-      <c r="L5">
-        <v>-0.831743348192543</v>
-      </c>
-      <c r="M5">
-        <v>8.349213213751526E-07</v>
-      </c>
-      <c r="N5">
-        <v>1.746329584159736E-07</v>
-      </c>
-      <c r="O5">
-        <v>0.1886743079377197</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15">
+      <c r="I5" s="2">
+        <v>5.4960097837528964E-3</v>
+      </c>
+      <c r="J5" s="2">
+        <v>8.1673297739886415E-3</v>
+      </c>
+      <c r="K5" s="2">
+        <v>3.4470869932094121E-4</v>
+      </c>
+      <c r="L5" s="2">
+        <v>-0.83174334819254303</v>
+      </c>
+      <c r="M5" s="2">
+        <v>8.3492132137515258E-7</v>
+      </c>
+      <c r="N5" s="2">
+        <v>1.746329584159736E-7</v>
+      </c>
+      <c r="O5" s="2">
+        <v>0.18867430793771969</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6">
-        <v>-0.0004272389117015966</v>
-      </c>
-      <c r="C6">
-        <v>0.3213107807895099</v>
-      </c>
-      <c r="D6">
-        <v>-0.006690812481156172</v>
-      </c>
-      <c r="E6">
-        <v>-0.0002147425614279354</v>
-      </c>
-      <c r="F6">
-        <v>0.001645162252369232</v>
-      </c>
-      <c r="G6">
-        <v>5.863997420889604E-06</v>
-      </c>
-      <c r="H6">
-        <v>-0.02453741277700528</v>
-      </c>
-      <c r="I6">
-        <v>0.002666926534053793</v>
-      </c>
-      <c r="J6">
-        <v>0.0007216756629232683</v>
-      </c>
-      <c r="K6">
-        <v>-9.344738362427031E-05</v>
-      </c>
-      <c r="L6">
-        <v>0.07818242673847832</v>
-      </c>
-      <c r="M6">
-        <v>6.180527819655973E-08</v>
-      </c>
-      <c r="N6">
-        <v>9.221371704434601E-09</v>
-      </c>
-      <c r="O6">
-        <v>0.0003380501501776491</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15">
+      <c r="B6" s="2">
+        <v>-4.2723891170159657E-4</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.32131078078950992</v>
+      </c>
+      <c r="D6" s="2">
+        <v>-6.6908124811561722E-3</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-2.1474256142793539E-4</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1.645162252369232E-3</v>
+      </c>
+      <c r="G6" s="2">
+        <v>5.8639974208896036E-6</v>
+      </c>
+      <c r="H6" s="2">
+        <v>-2.4537412777005281E-2</v>
+      </c>
+      <c r="I6" s="2">
+        <v>2.666926534053793E-3</v>
+      </c>
+      <c r="J6" s="2">
+        <v>7.2167566292326833E-4</v>
+      </c>
+      <c r="K6" s="2">
+        <v>-9.3447383624270305E-5</v>
+      </c>
+      <c r="L6" s="2">
+        <v>7.8182426738478319E-2</v>
+      </c>
+      <c r="M6" s="2">
+        <v>6.1805278196559732E-8</v>
+      </c>
+      <c r="N6" s="2">
+        <v>9.221371704434601E-9</v>
+      </c>
+      <c r="O6" s="2">
+        <v>3.3805015017764907E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7">
-        <v>-8.312614879468474E-06</v>
-      </c>
-      <c r="C7">
-        <v>0.0107748919153685</v>
-      </c>
-      <c r="D7">
-        <v>-3.046235227589717E-05</v>
-      </c>
-      <c r="E7">
-        <v>-0.0008843680115824424</v>
-      </c>
-      <c r="F7">
-        <v>5.863996738396824E-06</v>
-      </c>
-      <c r="G7">
-        <v>5.789062431163621E-07</v>
-      </c>
-      <c r="H7">
-        <v>-1.300337584035887E-05</v>
-      </c>
-      <c r="I7">
-        <v>5.014306187869823E-06</v>
-      </c>
-      <c r="J7">
-        <v>-2.797042397425519E-06</v>
-      </c>
-      <c r="K7">
-        <v>-5.177215420981011E-07</v>
-      </c>
-      <c r="L7">
-        <v>0.0008016473967512482</v>
-      </c>
-      <c r="M7">
-        <v>-3.019660185323107E-10</v>
-      </c>
-      <c r="N7">
-        <v>-7.836640095205464E-11</v>
-      </c>
-      <c r="O7">
-        <v>-0.0001181205734478254</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15">
+      <c r="B7" s="2">
+        <v>-8.3126148794684737E-6</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1.07748919153685E-2</v>
+      </c>
+      <c r="D7" s="2">
+        <v>-3.0462352275897171E-5</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-8.8436801158244243E-4</v>
+      </c>
+      <c r="F7" s="2">
+        <v>5.8639967383968238E-6</v>
+      </c>
+      <c r="G7" s="2">
+        <v>5.7890624311636207E-7</v>
+      </c>
+      <c r="H7" s="2">
+        <v>-1.300337584035887E-5</v>
+      </c>
+      <c r="I7" s="2">
+        <v>5.0143061878698233E-6</v>
+      </c>
+      <c r="J7" s="2">
+        <v>-2.7970423974255189E-6</v>
+      </c>
+      <c r="K7" s="2">
+        <v>-5.1772154209810107E-7</v>
+      </c>
+      <c r="L7" s="2">
+        <v>8.0164739675124823E-4</v>
+      </c>
+      <c r="M7" s="2">
+        <v>-3.0196601853231069E-10</v>
+      </c>
+      <c r="N7" s="2">
+        <v>-7.8366400952054641E-11</v>
+      </c>
+      <c r="O7" s="2">
+        <v>-1.181205734478254E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B8">
-        <v>0.003066538450151296</v>
-      </c>
-      <c r="C8">
-        <v>-3.469600305200435</v>
-      </c>
-      <c r="D8">
-        <v>0.07541907069017578</v>
-      </c>
-      <c r="E8">
+      <c r="B8" s="2">
+        <v>3.0665384501512962E-3</v>
+      </c>
+      <c r="C8" s="2">
+        <v>-3.4696003052004349</v>
+      </c>
+      <c r="D8" s="2">
+        <v>7.5419070690175782E-2</v>
+      </c>
+      <c r="E8" s="2">
         <v>-0.118073101907837</v>
       </c>
-      <c r="F8">
-        <v>-0.02453741306737393</v>
-      </c>
-      <c r="G8">
-        <v>-1.300338472472989E-05</v>
-      </c>
-      <c r="H8">
-        <v>0.4257248383098824</v>
-      </c>
-      <c r="I8">
-        <v>-0.03200915577015902</v>
-      </c>
-      <c r="J8">
-        <v>-0.00842946434361791</v>
-      </c>
-      <c r="K8">
-        <v>0.001026543395779972</v>
-      </c>
-      <c r="L8">
+      <c r="F8" s="2">
+        <v>-2.453741306737393E-2</v>
+      </c>
+      <c r="G8" s="2">
+        <v>-1.300338472472989E-5</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0.42572483830988239</v>
+      </c>
+      <c r="I8" s="2">
+        <v>-3.2009155770159017E-2</v>
+      </c>
+      <c r="J8" s="2">
+        <v>-8.4294643436179095E-3</v>
+      </c>
+      <c r="K8" s="2">
+        <v>1.0265433957799719E-3</v>
+      </c>
+      <c r="L8" s="2">
         <v>-1.022312045336405</v>
       </c>
-      <c r="M8">
-        <v>-1.189743370475536E-06</v>
-      </c>
-      <c r="N8">
-        <v>-1.684259836702912E-07</v>
-      </c>
-      <c r="O8">
-        <v>-0.01254391673624527</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15">
+      <c r="M8" s="2">
+        <v>-1.189743370475536E-6</v>
+      </c>
+      <c r="N8" s="2">
+        <v>-1.684259836702912E-7</v>
+      </c>
+      <c r="O8" s="2">
+        <v>-1.254391673624527E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9">
-        <v>-0.00410704941661557</v>
-      </c>
-      <c r="C9">
-        <v>-2.019188357881214</v>
-      </c>
-      <c r="D9">
-        <v>-0.4271095497186794</v>
-      </c>
-      <c r="E9">
-        <v>0.005495946116883276</v>
-      </c>
-      <c r="F9">
-        <v>0.00266692374474121</v>
-      </c>
-      <c r="G9">
-        <v>5.014336923793139E-06</v>
-      </c>
-      <c r="H9">
-        <v>-0.0320091062956882</v>
-      </c>
-      <c r="I9">
+      <c r="B9" s="2">
+        <v>-4.1070494166155699E-3</v>
+      </c>
+      <c r="C9" s="2">
+        <v>-2.0191883578812142</v>
+      </c>
+      <c r="D9" s="2">
+        <v>-0.42710954971867943</v>
+      </c>
+      <c r="E9" s="2">
+        <v>5.4959461168832763E-3</v>
+      </c>
+      <c r="F9" s="2">
+        <v>2.66692374474121E-3</v>
+      </c>
+      <c r="G9" s="2">
+        <v>5.0143369237931394E-6</v>
+      </c>
+      <c r="H9" s="2">
+        <v>-3.2009106295688199E-2</v>
+      </c>
+      <c r="I9" s="2">
         <v>0.2225199200101971</v>
       </c>
-      <c r="J9">
-        <v>0.002541848085790388</v>
-      </c>
-      <c r="K9">
-        <v>-0.005696413853777811</v>
-      </c>
-      <c r="L9">
-        <v>0.5499650331113967</v>
-      </c>
-      <c r="M9">
-        <v>-1.443401580909015E-06</v>
-      </c>
-      <c r="N9">
-        <v>4.088950345187541E-08</v>
-      </c>
-      <c r="O9">
-        <v>0.001929035104310978</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15">
+      <c r="J9" s="2">
+        <v>2.541848085790388E-3</v>
+      </c>
+      <c r="K9" s="2">
+        <v>-5.6964138537778106E-3</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0.54996503311139666</v>
+      </c>
+      <c r="M9" s="2">
+        <v>-1.443401580909015E-6</v>
+      </c>
+      <c r="N9" s="2">
+        <v>4.0889503451875409E-8</v>
+      </c>
+      <c r="O9" s="2">
+        <v>1.929035104310978E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B10">
-        <v>-0.0003301661603990506</v>
-      </c>
-      <c r="C10">
-        <v>0.0586693483008327</v>
-      </c>
-      <c r="D10">
-        <v>-0.00592612789480066</v>
-      </c>
-      <c r="E10">
-        <v>0.008167328787478372</v>
-      </c>
-      <c r="F10">
-        <v>0.0007216756684299712</v>
-      </c>
-      <c r="G10">
-        <v>-2.797041764467581E-06</v>
-      </c>
-      <c r="H10">
-        <v>-0.008429464147061751</v>
-      </c>
-      <c r="I10">
-        <v>0.002541850901285691</v>
-      </c>
-      <c r="J10">
-        <v>0.0006717413599097153</v>
-      </c>
-      <c r="K10">
-        <v>-8.296633106942738E-05</v>
-      </c>
-      <c r="L10">
-        <v>0.06617046624122599</v>
-      </c>
-      <c r="M10">
-        <v>5.768222596211136E-08</v>
-      </c>
-      <c r="N10">
-        <v>8.427430798018363E-09</v>
-      </c>
-      <c r="O10">
-        <v>0.001762220143555311</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15">
+      <c r="B10" s="2">
+        <v>-3.3016616039905061E-4</v>
+      </c>
+      <c r="C10" s="2">
+        <v>5.8669348300832702E-2</v>
+      </c>
+      <c r="D10" s="2">
+        <v>-5.9261278948006596E-3</v>
+      </c>
+      <c r="E10" s="2">
+        <v>8.1673287874783722E-3</v>
+      </c>
+      <c r="F10" s="2">
+        <v>7.2167566842997117E-4</v>
+      </c>
+      <c r="G10" s="2">
+        <v>-2.7970417644675812E-6</v>
+      </c>
+      <c r="H10" s="2">
+        <v>-8.429464147061751E-3</v>
+      </c>
+      <c r="I10" s="2">
+        <v>2.5418509012856911E-3</v>
+      </c>
+      <c r="J10" s="2">
+        <v>6.7174135990971532E-4</v>
+      </c>
+      <c r="K10" s="2">
+        <v>-8.2966331069427384E-5</v>
+      </c>
+      <c r="L10" s="2">
+        <v>6.6170466241225995E-2</v>
+      </c>
+      <c r="M10" s="2">
+        <v>5.7682225962111362E-8</v>
+      </c>
+      <c r="N10" s="2">
+        <v>8.4274307980183631E-9</v>
+      </c>
+      <c r="O10" s="2">
+        <v>1.762220143555311E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B11">
-        <v>0.0002184840621661411</v>
-      </c>
-      <c r="C11">
-        <v>0.03054754517637611</v>
-      </c>
-      <c r="D11">
-        <v>0.01244898474251793</v>
-      </c>
-      <c r="E11">
-        <v>0.0003447105522423924</v>
-      </c>
-      <c r="F11">
-        <v>-9.344729924215692E-05</v>
-      </c>
-      <c r="G11">
-        <v>-5.177224262779219E-07</v>
-      </c>
-      <c r="H11">
-        <v>0.001026541917811745</v>
-      </c>
-      <c r="I11">
-        <v>-0.005696413673496587</v>
-      </c>
-      <c r="J11">
-        <v>-8.296624624199905E-05</v>
-      </c>
-      <c r="K11">
-        <v>0.0001656083480028601</v>
-      </c>
-      <c r="L11">
-        <v>-0.02219980500410423</v>
-      </c>
-      <c r="M11">
-        <v>4.207248975225549E-08</v>
-      </c>
-      <c r="N11">
-        <v>-1.746995647983719E-09</v>
-      </c>
-      <c r="O11">
-        <v>-1.36077554522489E-05</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15">
+      <c r="B11" s="2">
+        <v>2.1848406216614109E-4</v>
+      </c>
+      <c r="C11" s="2">
+        <v>3.054754517637611E-2</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1.2448984742517931E-2</v>
+      </c>
+      <c r="E11" s="2">
+        <v>3.4471055224239241E-4</v>
+      </c>
+      <c r="F11" s="2">
+        <v>-9.3447299242156921E-5</v>
+      </c>
+      <c r="G11" s="2">
+        <v>-5.1772242627792185E-7</v>
+      </c>
+      <c r="H11" s="2">
+        <v>1.026541917811745E-3</v>
+      </c>
+      <c r="I11" s="2">
+        <v>-5.6964136734965866E-3</v>
+      </c>
+      <c r="J11" s="2">
+        <v>-8.2966246241999045E-5</v>
+      </c>
+      <c r="K11" s="2">
+        <v>1.6560834800286009E-4</v>
+      </c>
+      <c r="L11" s="2">
+        <v>-2.219980500410423E-2</v>
+      </c>
+      <c r="M11" s="2">
+        <v>4.2072489752255488E-8</v>
+      </c>
+      <c r="N11" s="2">
+        <v>-1.7469956479837191E-9</v>
+      </c>
+      <c r="O11" s="2">
+        <v>-1.3607755452248901E-5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B12">
-        <v>-0.08935808811995211</v>
-      </c>
-      <c r="C12">
-        <v>180.7472244134096</v>
-      </c>
-      <c r="D12">
+      <c r="B12" s="2">
+        <v>-8.9358088119952106E-2</v>
+      </c>
+      <c r="C12" s="2">
+        <v>180.74722441340961</v>
+      </c>
+      <c r="D12" s="2">
         <v>-1.585901204450874</v>
       </c>
-      <c r="E12">
-        <v>-0.8317434937895108</v>
-      </c>
-      <c r="F12">
-        <v>0.07818242690730622</v>
-      </c>
-      <c r="G12">
-        <v>0.0008016474883183874</v>
-      </c>
-      <c r="H12">
+      <c r="E12" s="2">
+        <v>-0.83174349378951085</v>
+      </c>
+      <c r="F12" s="2">
+        <v>7.8182426907306216E-2</v>
+      </c>
+      <c r="G12" s="2">
+        <v>8.0164748831838741E-4</v>
+      </c>
+      <c r="H12" s="2">
         <v>-1.022312013594515</v>
       </c>
-      <c r="I12">
-        <v>0.5499653623475809</v>
-      </c>
-      <c r="J12">
-        <v>0.06617046551115799</v>
-      </c>
-      <c r="K12">
-        <v>-0.02219981522299294</v>
-      </c>
-      <c r="L12">
-        <v>161.7925889634901</v>
-      </c>
-      <c r="M12">
-        <v>0.0001085230187175703</v>
-      </c>
-      <c r="N12">
-        <v>4.737477031584279E-06</v>
-      </c>
-      <c r="O12">
-        <v>-0.0642863521346738</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
+      <c r="I12" s="2">
+        <v>0.54996536234758087</v>
+      </c>
+      <c r="J12" s="2">
+        <v>6.6170465511157989E-2</v>
+      </c>
+      <c r="K12" s="2">
+        <v>-2.2199815222992941E-2</v>
+      </c>
+      <c r="L12" s="2">
+        <v>161.79258896349009</v>
+      </c>
+      <c r="M12" s="2">
+        <v>1.085230187175703E-4</v>
+      </c>
+      <c r="N12" s="2">
+        <v>4.7374770315842793E-6</v>
+      </c>
+      <c r="O12" s="2">
+        <v>-6.4286352134673805E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B13">
-        <v>1.81897298319865E-08</v>
-      </c>
-      <c r="C13">
-        <v>0.0001281684801629818</v>
-      </c>
-      <c r="D13">
-        <v>3.259375693301747E-06</v>
-      </c>
-      <c r="E13">
-        <v>8.349217725570104E-07</v>
-      </c>
-      <c r="F13">
-        <v>6.180534542525135E-08</v>
-      </c>
-      <c r="G13">
-        <v>-3.019660836334935E-10</v>
-      </c>
-      <c r="H13">
-        <v>-1.189744278363214E-06</v>
-      </c>
-      <c r="I13">
-        <v>-1.443398860038581E-06</v>
-      </c>
-      <c r="J13">
-        <v>5.768228835652867E-08</v>
-      </c>
-      <c r="K13">
-        <v>4.207241161185047E-08</v>
-      </c>
-      <c r="L13">
-        <v>0.0001085230265569252</v>
-      </c>
-      <c r="M13">
+      <c r="B13" s="2">
+        <v>1.8189729831986501E-8</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1.2816848016298179E-4</v>
+      </c>
+      <c r="D13" s="2">
+        <v>3.2593756933017469E-6</v>
+      </c>
+      <c r="E13" s="2">
+        <v>8.3492177255701039E-7</v>
+      </c>
+      <c r="F13" s="2">
+        <v>6.1805345425251353E-8</v>
+      </c>
+      <c r="G13" s="2">
+        <v>-3.0196608363349352E-10</v>
+      </c>
+      <c r="H13" s="2">
+        <v>-1.189744278363214E-6</v>
+      </c>
+      <c r="I13" s="2">
+        <v>-1.443398860038581E-6</v>
+      </c>
+      <c r="J13" s="2">
+        <v>5.7682288356528667E-8</v>
+      </c>
+      <c r="K13" s="2">
+        <v>4.2072411611850467E-8</v>
+      </c>
+      <c r="L13" s="2">
+        <v>1.085230265569252E-4</v>
+      </c>
+      <c r="M13" s="2">
         <v>1.373051010260969E-10</v>
       </c>
-      <c r="N13">
-        <v>9.680720496739259E-12</v>
-      </c>
-      <c r="O13">
-        <v>9.761699095830684E-08</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15">
+      <c r="N13" s="2">
+        <v>9.6807204967392587E-12</v>
+      </c>
+      <c r="O13" s="2">
+        <v>9.7616990958306842E-8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B14">
-        <v>3.144338194957824E-09</v>
-      </c>
-      <c r="C14">
-        <v>1.688883549682678E-06</v>
-      </c>
-      <c r="D14">
-        <v>-1.419652918313414E-07</v>
-      </c>
-      <c r="E14">
-        <v>1.746329266277113E-07</v>
-      </c>
-      <c r="F14">
-        <v>9.221376385701814E-09</v>
-      </c>
-      <c r="G14">
-        <v>-7.83663660864183E-11</v>
-      </c>
-      <c r="H14">
-        <v>-1.684260298315625E-07</v>
-      </c>
-      <c r="I14">
-        <v>4.088985615872569E-08</v>
-      </c>
-      <c r="J14">
-        <v>8.427434833999732E-09</v>
-      </c>
-      <c r="K14">
-        <v>-1.74700602172339E-09</v>
-      </c>
-      <c r="L14">
-        <v>4.7374775265477E-06</v>
-      </c>
-      <c r="M14">
-        <v>9.680716541707693E-12</v>
-      </c>
-      <c r="N14">
+      <c r="B14" s="2">
+        <v>3.144338194957824E-9</v>
+      </c>
+      <c r="C14" s="2">
+        <v>1.688883549682678E-6</v>
+      </c>
+      <c r="D14" s="2">
+        <v>-1.4196529183134141E-7</v>
+      </c>
+      <c r="E14" s="2">
+        <v>1.7463292662771131E-7</v>
+      </c>
+      <c r="F14" s="2">
+        <v>9.2213763857018137E-9</v>
+      </c>
+      <c r="G14" s="2">
+        <v>-7.8366366086418304E-11</v>
+      </c>
+      <c r="H14" s="2">
+        <v>-1.684260298315625E-7</v>
+      </c>
+      <c r="I14" s="2">
+        <v>4.0889856158725687E-8</v>
+      </c>
+      <c r="J14" s="2">
+        <v>8.4274348339997317E-9</v>
+      </c>
+      <c r="K14" s="2">
+        <v>-1.7470060217233901E-9</v>
+      </c>
+      <c r="L14" s="2">
+        <v>4.7374775265476999E-6</v>
+      </c>
+      <c r="M14" s="2">
+        <v>9.6807165417076929E-12</v>
+      </c>
+      <c r="N14" s="2">
         <v>1.295355820006276E-12</v>
       </c>
-      <c r="O14">
-        <v>2.116655151366869E-08</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15">
+      <c r="O14" s="2">
+        <v>2.1166551513668691E-8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B15">
-        <v>0.0009022317840168874</v>
-      </c>
-      <c r="C15">
+      <c r="B15" s="2">
+        <v>9.0223178401688741E-4</v>
+      </c>
+      <c r="C15" s="2">
         <v>-1.759378859458596</v>
       </c>
-      <c r="D15">
-        <v>-0.002079110383161237</v>
-      </c>
-      <c r="E15">
-        <v>0.1886743073290648</v>
-      </c>
-      <c r="F15">
-        <v>0.0003380502652809771</v>
-      </c>
-      <c r="G15">
-        <v>-0.0001181205726982876</v>
-      </c>
-      <c r="H15">
-        <v>-0.0125439179162168</v>
-      </c>
-      <c r="I15">
-        <v>0.001929043341876873</v>
-      </c>
-      <c r="J15">
-        <v>0.00176222024436801</v>
-      </c>
-      <c r="K15">
-        <v>-1.360799685134756E-05</v>
-      </c>
-      <c r="L15">
-        <v>-0.06428633618282456</v>
-      </c>
-      <c r="M15">
-        <v>9.761690682507365E-08</v>
-      </c>
-      <c r="N15">
-        <v>2.116655226542033E-08</v>
-      </c>
-      <c r="O15">
-        <v>0.02739900398013492</v>
+      <c r="D15" s="2">
+        <v>-2.079110383161237E-3</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0.18867430732906479</v>
+      </c>
+      <c r="F15" s="2">
+        <v>3.3805026528097709E-4</v>
+      </c>
+      <c r="G15" s="2">
+        <v>-1.181205726982876E-4</v>
+      </c>
+      <c r="H15" s="2">
+        <v>-1.25439179162168E-2</v>
+      </c>
+      <c r="I15" s="2">
+        <v>1.929043341876873E-3</v>
+      </c>
+      <c r="J15" s="2">
+        <v>1.7622202443680101E-3</v>
+      </c>
+      <c r="K15" s="2">
+        <v>-1.360799685134756E-5</v>
+      </c>
+      <c r="L15" s="2">
+        <v>-6.4286336182824561E-2</v>
+      </c>
+      <c r="M15" s="2">
+        <v>9.7616906825073654E-8</v>
+      </c>
+      <c r="N15" s="2">
+        <v>2.1166552265420331E-8</v>
+      </c>
+      <c r="O15" s="2">
+        <v>2.7399003980134919E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1851,24 +1868,24 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.07428864793095931</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>7.4288647930959309E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1876,71 +1893,71 @@
         <v>60.26001475393506</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.9730098655775894</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
+        <v>0.97300986557758939</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1.183106933476142</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>1.1831069334761419</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.04056059975356913</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+        <v>4.0560599753569133E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.0007608588851530631</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
+        <v>7.6085888515306315E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.6524759292953897</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
+        <v>0.65247592929538967</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.4717201712988296</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
+        <v>0.47172017129882959</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.02591797368448612</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
+        <v>2.5917973684486121E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.0128688907059956</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
+        <v>1.28688907059956E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1948,28 +1965,28 @@
         <v>12.71977157670255</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B13">
-        <v>1.171772593236831E-05</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
+        <v>1.171772593236831E-5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B14">
-        <v>1.13813699527178E-06</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
+        <v>1.1381369952717801E-6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.1655264449570971</v>
+        <v>0.16552644495709709</v>
       </c>
     </row>
   </sheetData>
@@ -1978,11 +1995,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
@@ -1993,12 +2010,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>8.804925053332726</v>
+        <v>8.8049250533327257</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -2007,49 +2024,49 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.4899275059345551</v>
+        <v>0.48992750593455509</v>
       </c>
       <c r="C3">
-        <v>0.6241987055102443</v>
+        <v>0.62419870551024426</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>5.436574598781578</v>
+        <v>5.4365745987815783</v>
       </c>
       <c r="C4">
-        <v>5.592443219626375E-08</v>
+        <v>5.5924432196263751E-8</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>4.148556656764785</v>
+        <v>4.1485566567647849</v>
       </c>
       <c r="C5">
-        <v>3.380595918334173E-05</v>
+        <v>3.3805959183341727E-5</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2063,7 +2080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -2071,13 +2088,13 @@
         <v>3.601835243378031</v>
       </c>
       <c r="C7">
-        <v>0.0003179048696002607</v>
+        <v>3.1790486960026071E-4</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -2091,21 +2108,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9">
-        <v>6.92665419607431</v>
+        <v>6.9266541960743098</v>
       </c>
       <c r="C9">
-        <v>4.644729045821805E-12</v>
+        <v>4.6447290458218049E-12</v>
       </c>
       <c r="D9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -2119,40 +2136,40 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B11">
-        <v>6.216542033629058</v>
+        <v>6.2165420336290582</v>
       </c>
       <c r="C11">
-        <v>5.338436359636489E-10</v>
+        <v>5.3384363596364892E-10</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B12">
-        <v>1.681148119494352</v>
+        <v>1.6811481194943521</v>
       </c>
       <c r="C12">
-        <v>0.09277339356623693</v>
+        <v>9.2773393566236928E-2</v>
       </c>
       <c r="D12" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B13">
-        <v>1.155925187731533</v>
+        <v>1.1559251877315331</v>
       </c>
       <c r="C13">
         <v>0.2477464650218191</v>
@@ -2161,26 +2178,26 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B14">
-        <v>1.953886144199568</v>
+        <v>1.9538861441995681</v>
       </c>
       <c r="C14">
-        <v>0.05074966924742164</v>
+        <v>5.0749669247421643E-2</v>
       </c>
       <c r="D14" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B15">
-        <v>48.10847258357437</v>
+        <v>48.108472583574368</v>
       </c>
       <c r="C15">
         <v>0</v>

</xml_diff>

<commit_message>
Update (polish) of agriAcoDM.mo
</commit_message>
<xml_diff>
--- a/Parameter_estimation/uit_real_R2+batch_april24_FIM_COV_sigma_01-12-2025.xlsx
+++ b/Parameter_estimation/uit_real_R2+batch_april24_FIM_COV_sigma_01-12-2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10530006_polimi_it/Documents/Work_cloud/DOTTORATO/Modelling/Pilot_plant/Parameter_estimation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_ED70979F7DD2020A4F50F93CA6B0D01A6D9808E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01D1213C-6F0F-48E6-9675-E4EB344A8D05}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_48A9D0DC0887C130A1F2F83CA6B0D0D3EDDC2F08" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05CDEC65-8670-479A-B43A-48452C9F5CDA}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FIM" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
     <sheet name="Parameter_Std_Dev" sheetId="3" r:id="rId3"/>
     <sheet name="Parameter_Significance" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -135,12 +148,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -497,46 +509,46 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>41721207236.313347</v>
+        <v>5464725092256.6338</v>
       </c>
       <c r="C2">
-        <v>3493080.1264431579</v>
+        <v>457530447.48001528</v>
       </c>
       <c r="D2">
-        <v>34549075388.481239</v>
+        <v>4525305275092.1006</v>
       </c>
       <c r="E2">
-        <v>109684106.4474176</v>
+        <v>14366638178.27519</v>
       </c>
       <c r="F2">
-        <v>-473890193.09389907</v>
+        <v>-62071061714.641937</v>
       </c>
       <c r="G2">
-        <v>76297121892.758575</v>
+        <v>9993545827011.0078</v>
       </c>
       <c r="H2">
-        <v>699544.90798796399</v>
+        <v>91627756.363552064</v>
       </c>
       <c r="I2">
-        <v>-2325588.4294158439</v>
+        <v>-304610108.05624652</v>
       </c>
       <c r="J2">
-        <v>135.6478942481034</v>
+        <v>17767.425741319159</v>
       </c>
       <c r="K2">
-        <v>-2359621312976.292</v>
+        <v>-309067801518979.13</v>
       </c>
       <c r="L2">
-        <v>402336557.03475672</v>
+        <v>52698826913.289948</v>
       </c>
       <c r="M2">
-        <v>-750708030461507.75</v>
+        <v>-9.8329201928051984E+16</v>
       </c>
       <c r="N2">
-        <v>4631802344998073</v>
+        <v>6.0668250450464947E+17</v>
       </c>
       <c r="O2">
-        <v>-79438170.225813538</v>
+        <v>-10404966463.62903</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -544,46 +556,46 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>3493080.1264431579</v>
+        <v>457530447.48001528</v>
       </c>
       <c r="C3">
-        <v>292.45827561727708</v>
+        <v>38306.755318738578</v>
       </c>
       <c r="D3">
-        <v>2892598.1956092739</v>
+        <v>378878153.06561708</v>
       </c>
       <c r="E3">
-        <v>9233.603082187803</v>
+        <v>1209435.339906733</v>
       </c>
       <c r="F3">
-        <v>-39732.165553595332</v>
+        <v>-5204196.5334465504</v>
       </c>
       <c r="G3">
-        <v>6456339.2001612857</v>
+        <v>845663900.16951895</v>
       </c>
       <c r="H3">
-        <v>69.982492767792863</v>
+        <v>9166.443388866317</v>
       </c>
       <c r="I3">
-        <v>-194.65344226594561</v>
+        <v>-25496.087498613721</v>
       </c>
       <c r="J3">
-        <v>-4.8989314866936349</v>
+        <v>-641.67160046317065</v>
       </c>
       <c r="K3">
-        <v>-197557710.13710821</v>
+        <v>-25876494168.542561</v>
       </c>
       <c r="L3">
-        <v>33685.361610551357</v>
+        <v>4412174.3599666869</v>
       </c>
       <c r="M3">
-        <v>-62852531697.982117</v>
+        <v>-8232547182452.2607</v>
       </c>
       <c r="N3">
-        <v>387794580488.62549</v>
+        <v>50794090464209.359</v>
       </c>
       <c r="O3">
-        <v>-6696.4673795275576</v>
+        <v>-877116.35742244858</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -591,46 +603,46 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>34549075388.481239</v>
+        <v>4525305275092.1006</v>
       </c>
       <c r="C4">
-        <v>2892598.1956092739</v>
+        <v>378878153.06561708</v>
       </c>
       <c r="D4">
-        <v>28609878188.30407</v>
+        <v>3747377642657.2622</v>
       </c>
       <c r="E4">
-        <v>90828594.161216363</v>
+        <v>11896906405.31554</v>
       </c>
       <c r="F4">
-        <v>-392425987.97591043</v>
+        <v>-51400721249.480659</v>
       </c>
       <c r="G4">
-        <v>63180953895.488258</v>
+        <v>8275564562400.0723</v>
       </c>
       <c r="H4">
-        <v>579233.82926844526</v>
+        <v>75869176.631401598</v>
       </c>
       <c r="I4">
-        <v>-1924911.5677244889</v>
+        <v>-252128671.27592209</v>
       </c>
       <c r="J4">
-        <v>1007.3856186226531</v>
+        <v>131949.33302107709</v>
       </c>
       <c r="K4">
-        <v>-1953987924483.7271</v>
+        <v>-255937149191568.59</v>
       </c>
       <c r="L4">
-        <v>333172488.51937211</v>
+        <v>43639582329.168533</v>
       </c>
       <c r="M4">
-        <v>-621656812714365.38</v>
+        <v>-8.1425821740259488E+16</v>
       </c>
       <c r="N4">
-        <v>3835567713062442</v>
+        <v>5.0239013952545088E+17</v>
       </c>
       <c r="O4">
-        <v>-65782311.962163098</v>
+        <v>-8616295515.3752079</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -638,46 +650,46 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>109684106.4474176</v>
+        <v>14366638178.27519</v>
       </c>
       <c r="C5">
-        <v>9233.603082187803</v>
+        <v>1209435.339906733</v>
       </c>
       <c r="D5">
-        <v>90828594.161216363</v>
+        <v>11896906405.31554</v>
       </c>
       <c r="E5">
-        <v>1472104.2689854889</v>
+        <v>192819088.1816383</v>
       </c>
       <c r="F5">
-        <v>-2575781.1819089469</v>
+        <v>-337380842.72616261</v>
       </c>
       <c r="G5">
-        <v>1809313062.638026</v>
+        <v>236987353629.1134</v>
       </c>
       <c r="H5">
-        <v>269361.24895347352</v>
+        <v>35281461.720418394</v>
       </c>
       <c r="I5">
-        <v>-5983.913224349104</v>
+        <v>-783784.62449008436</v>
       </c>
       <c r="J5">
-        <v>-116378.5110605714</v>
+        <v>-15243484.35053502</v>
       </c>
       <c r="K5">
-        <v>-6203372990.3741322</v>
+        <v>-812529892654.1825</v>
       </c>
       <c r="L5">
-        <v>1057746.280846549</v>
+        <v>138545670.7770482</v>
       </c>
       <c r="M5">
-        <v>-1973591735056.9719</v>
+        <v>-258504894533563.81</v>
       </c>
       <c r="N5">
-        <v>12176949940661.93</v>
+        <v>1594960651808987</v>
       </c>
       <c r="O5">
-        <v>-1275313.6268447719</v>
+        <v>-167043066.07526791</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -685,46 +697,46 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>-473890193.09389907</v>
+        <v>-62071061714.641937</v>
       </c>
       <c r="C6">
-        <v>-39732.165553595332</v>
+        <v>-5204196.5334465504</v>
       </c>
       <c r="D6">
-        <v>-392425987.97591043</v>
+        <v>-51400721249.480659</v>
       </c>
       <c r="E6">
-        <v>-2575781.1819089469</v>
+        <v>-337380842.72616261</v>
       </c>
       <c r="F6">
-        <v>6953347.9784761025</v>
+        <v>910763079.26433718</v>
       </c>
       <c r="G6">
-        <v>-2677254971.609931</v>
+        <v>-350672077604.49298</v>
       </c>
       <c r="H6">
-        <v>-304922.99107377842</v>
+        <v>-39939408.059038348</v>
       </c>
       <c r="I6">
-        <v>25733.42390021863</v>
+        <v>3370614.050084414</v>
       </c>
       <c r="J6">
-        <v>110348.14009798539</v>
+        <v>14453614.600884611</v>
       </c>
       <c r="K6">
-        <v>26801729608.2603</v>
+        <v>3510542815229.4229</v>
       </c>
       <c r="L6">
-        <v>-4569987.3525162106</v>
+        <v>-598585856.23222673</v>
       </c>
       <c r="M6">
-        <v>8526981373949.2637</v>
+        <v>1116880650444549</v>
       </c>
       <c r="N6">
-        <v>-52610754075114.672</v>
+        <v>-6891059174974799</v>
       </c>
       <c r="O6">
-        <v>2088542.5451891101</v>
+        <v>273561375.83206213</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -732,46 +744,46 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>76297121892.758575</v>
+        <v>9993545827011.0078</v>
       </c>
       <c r="C7">
-        <v>6456339.2001612866</v>
+        <v>845663900.16951907</v>
       </c>
       <c r="D7">
-        <v>63180953895.488258</v>
+        <v>8275564562400.0723</v>
       </c>
       <c r="E7">
-        <v>1809313062.638026</v>
+        <v>236987353629.1134</v>
       </c>
       <c r="F7">
-        <v>-2677254971.609931</v>
+        <v>-350672077604.49298</v>
       </c>
       <c r="G7">
-        <v>2325994330108.8091</v>
+        <v>304663273720634.88</v>
       </c>
       <c r="H7">
-        <v>364694421.15641111</v>
+        <v>47768386542.871132</v>
       </c>
       <c r="I7">
-        <v>-4101154.7952557132</v>
+        <v>-537177253.52289915</v>
       </c>
       <c r="J7">
-        <v>-157698594.56077081</v>
+        <v>-20655669473.527908</v>
       </c>
       <c r="K7">
-        <v>-4315102561936.3389</v>
+        <v>-565200549262871.63</v>
       </c>
       <c r="L7">
-        <v>735783060.07864702</v>
+        <v>96374300199.287598</v>
       </c>
       <c r="M7">
-        <v>-1372840925738698</v>
+        <v>-1.7981738189088922E+17</v>
       </c>
       <c r="N7">
-        <v>8470393066992937</v>
+        <v>1.109468603635812E+18</v>
       </c>
       <c r="O7">
-        <v>-1593910278.227237</v>
+        <v>-208773476829.13821</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -779,46 +791,46 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>699544.90798796399</v>
+        <v>91627756.363552064</v>
       </c>
       <c r="C8">
-        <v>69.982492767792863</v>
+        <v>9166.443388866317</v>
       </c>
       <c r="D8">
-        <v>579233.82926844526</v>
+        <v>75869176.631401598</v>
       </c>
       <c r="E8">
-        <v>269361.24895347352</v>
+        <v>35281461.720418394</v>
       </c>
       <c r="F8">
-        <v>-304922.99107377842</v>
+        <v>-39939408.059038348</v>
       </c>
       <c r="G8">
-        <v>364694421.15641111</v>
+        <v>47768386542.871117</v>
       </c>
       <c r="H8">
-        <v>60641.734198307429</v>
+        <v>7942972.6142490879</v>
       </c>
       <c r="I8">
-        <v>-29.599678823348359</v>
+        <v>-3877.0236602334298</v>
       </c>
       <c r="J8">
-        <v>-27213.250071009759</v>
+        <v>-3564444.5680245021</v>
       </c>
       <c r="K8">
-        <v>-39560026.106641062</v>
+        <v>-5181649372.962676</v>
       </c>
       <c r="L8">
-        <v>6747.5448319880034</v>
+        <v>883806.58176155167</v>
       </c>
       <c r="M8">
-        <v>-12583903663.96908</v>
+        <v>-1648264244165.447</v>
       </c>
       <c r="N8">
-        <v>77657865526.522308</v>
+        <v>10171778682005.789</v>
       </c>
       <c r="O8">
-        <v>-242910.15354982379</v>
+        <v>-31816845.65714718</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -826,46 +838,46 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>-2325588.4294158439</v>
+        <v>-304610108.05624652</v>
       </c>
       <c r="C9">
-        <v>-194.65344226594561</v>
+        <v>-25496.087498613721</v>
       </c>
       <c r="D9">
-        <v>-1924911.5677244889</v>
+        <v>-252128671.27592209</v>
       </c>
       <c r="E9">
-        <v>-5983.913224349104</v>
+        <v>-783784.62449008436</v>
       </c>
       <c r="F9">
-        <v>25733.42390021863</v>
+        <v>3370614.050084414</v>
       </c>
       <c r="G9">
-        <v>-4101154.7952557132</v>
+        <v>-537177253.52289915</v>
       </c>
       <c r="H9">
-        <v>-29.599678823348349</v>
+        <v>-3877.0236602334289</v>
       </c>
       <c r="I9">
-        <v>965.01779955614541</v>
+        <v>126399.9134502212</v>
       </c>
       <c r="J9">
-        <v>848.57088785610881</v>
+        <v>111147.469850528</v>
       </c>
       <c r="K9">
-        <v>131526117.8309859</v>
+        <v>17227547427.546669</v>
       </c>
       <c r="L9">
-        <v>-22375.83598448581</v>
+        <v>-2930830.6366123138</v>
       </c>
       <c r="M9">
-        <v>41752650917.457153</v>
+        <v>5468843646937.1396</v>
       </c>
       <c r="N9">
-        <v>-257609934187.74261</v>
+        <v>-33742251593933.809</v>
       </c>
       <c r="O9">
-        <v>4164.2213266783574</v>
+        <v>545437.83080664917</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -873,46 +885,46 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>135.6478942481034</v>
+        <v>17767.425741319159</v>
       </c>
       <c r="C10">
-        <v>-4.8989314866936358</v>
+        <v>-641.67160046317076</v>
       </c>
       <c r="D10">
-        <v>1007.3856186226531</v>
+        <v>131949.33302107709</v>
       </c>
       <c r="E10">
-        <v>-116378.5110605715</v>
+        <v>-15243484.35053502</v>
       </c>
       <c r="F10">
-        <v>110348.14009798539</v>
+        <v>14453614.600884611</v>
       </c>
       <c r="G10">
-        <v>-157698594.56077081</v>
+        <v>-20655669473.527908</v>
       </c>
       <c r="H10">
-        <v>-27213.250071009759</v>
+        <v>-3564444.5680245012</v>
       </c>
       <c r="I10">
-        <v>848.5708878561087</v>
+        <v>111147.469850528</v>
       </c>
       <c r="J10">
-        <v>23431.67508993734</v>
+        <v>3069126.501836577</v>
       </c>
       <c r="K10">
-        <v>-4135.448299562292</v>
+        <v>-541669.08359924611</v>
       </c>
       <c r="L10">
-        <v>55.635090778575503</v>
+        <v>7287.1926947270786</v>
       </c>
       <c r="M10">
-        <v>-106514360.9282804</v>
+        <v>-13951458728.25629</v>
       </c>
       <c r="N10">
-        <v>618226858.04161501</v>
+        <v>80976559587.817093</v>
       </c>
       <c r="O10">
-        <v>105944.69571676719</v>
+        <v>13876842.86784005</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -920,46 +932,46 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>-2359621312976.292</v>
+        <v>-309067801518979.13</v>
       </c>
       <c r="C11">
-        <v>-197557710.13710821</v>
+        <v>-25876494168.542561</v>
       </c>
       <c r="D11">
-        <v>-1953987924483.7271</v>
+        <v>-255937149191568.59</v>
       </c>
       <c r="E11">
-        <v>-6203372990.3741331</v>
+        <v>-812529892654.18262</v>
       </c>
       <c r="F11">
-        <v>26801729608.2603</v>
+        <v>3510542815229.4229</v>
       </c>
       <c r="G11">
-        <v>-4315102561936.3389</v>
+        <v>-565200549262871.63</v>
       </c>
       <c r="H11">
-        <v>-39560026.106641047</v>
+        <v>-5181649372.9626751</v>
       </c>
       <c r="I11">
-        <v>131526117.8309859</v>
+        <v>17227547427.546669</v>
       </c>
       <c r="J11">
-        <v>-4135.448299562292</v>
+        <v>-541669.08359924611</v>
       </c>
       <c r="K11">
-        <v>133452820228690.2</v>
+        <v>1.747991066522597E+16</v>
       </c>
       <c r="L11">
-        <v>-22754900629.555599</v>
+        <v>-2980481263109.459</v>
       </c>
       <c r="M11">
-        <v>4.2457704463027032E+16</v>
+        <v>5.5611929353946102E+18</v>
       </c>
       <c r="N11">
-        <v>-2.6196029237808518E+17</v>
+        <v>-3.4312069994164031E+19</v>
       </c>
       <c r="O11">
-        <v>4492759863.6256037</v>
+        <v>588470449121.35229</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -967,46 +979,46 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>402336557.03475672</v>
+        <v>52698826913.289948</v>
       </c>
       <c r="C12">
-        <v>33685.361610551357</v>
+        <v>4412174.3599666869</v>
       </c>
       <c r="D12">
-        <v>333172488.51937211</v>
+        <v>43639582329.168533</v>
       </c>
       <c r="E12">
-        <v>1057746.280846549</v>
+        <v>138545670.7770482</v>
       </c>
       <c r="F12">
-        <v>-4569987.3525162106</v>
+        <v>-598585856.23222673</v>
       </c>
       <c r="G12">
-        <v>735783060.07864702</v>
+        <v>96374300199.287598</v>
       </c>
       <c r="H12">
-        <v>6747.5448319880024</v>
+        <v>883806.58176155156</v>
       </c>
       <c r="I12">
-        <v>-22375.83598448581</v>
+        <v>-2930830.6366123138</v>
       </c>
       <c r="J12">
-        <v>55.635090778575503</v>
+        <v>7287.1926947270786</v>
       </c>
       <c r="K12">
-        <v>-22754900629.555599</v>
+        <v>-2980481263109.459</v>
       </c>
       <c r="L12">
-        <v>3879917.4745140998</v>
+        <v>508199157.77527589</v>
       </c>
       <c r="M12">
-        <v>-7239424538496.9023</v>
+        <v>-948233945028054.5</v>
       </c>
       <c r="N12">
-        <v>44666610930788.688</v>
+        <v>5850519812549753</v>
       </c>
       <c r="O12">
-        <v>-766080.2506618374</v>
+        <v>-100342685.3101752</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1014,46 +1026,46 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>-750708030461507.75</v>
+        <v>-9.8329201928051984E+16</v>
       </c>
       <c r="C13">
-        <v>-62852531697.982117</v>
+        <v>-8232547182452.2607</v>
       </c>
       <c r="D13">
-        <v>-621656812714365.38</v>
+        <v>-8.1425821740259488E+16</v>
       </c>
       <c r="E13">
-        <v>-1973591735056.9719</v>
+        <v>-258504894533563.81</v>
       </c>
       <c r="F13">
-        <v>8526981373949.2646</v>
+        <v>1116880650444549</v>
       </c>
       <c r="G13">
-        <v>-1372840925738698</v>
+        <v>-1.7981738189088922E+17</v>
       </c>
       <c r="H13">
-        <v>-12583903663.96908</v>
+        <v>-1648264244165.447</v>
       </c>
       <c r="I13">
-        <v>41752650917.457153</v>
+        <v>5468843646937.1396</v>
       </c>
       <c r="J13">
-        <v>-106514360.9282804</v>
+        <v>-13951458728.25629</v>
       </c>
       <c r="K13">
-        <v>4.2457704463027032E+16</v>
+        <v>5.5611929353946102E+18</v>
       </c>
       <c r="L13">
-        <v>-7239424538496.9023</v>
+        <v>-948233945028054.5</v>
       </c>
       <c r="M13">
-        <v>1.3507830546071491E+19</v>
+        <v>1.769281989108382E+21</v>
       </c>
       <c r="N13">
-        <v>-8.33421232053171E+19</v>
+        <v>-1.0916313838724019E+22</v>
       </c>
       <c r="O13">
-        <v>1429381826137.4431</v>
+        <v>187223219296257.41</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1061,46 +1073,46 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>4631802344998073</v>
+        <v>6.0668250450464947E+17</v>
       </c>
       <c r="C14">
-        <v>387794580488.62549</v>
+        <v>50794090464209.359</v>
       </c>
       <c r="D14">
-        <v>3835567713062442</v>
+        <v>5.0239013952545088E+17</v>
       </c>
       <c r="E14">
-        <v>12176949940661.93</v>
+        <v>1594960651808987</v>
       </c>
       <c r="F14">
-        <v>-52610754075114.672</v>
+        <v>-6891059174974799</v>
       </c>
       <c r="G14">
-        <v>8470393066992937</v>
+        <v>1.109468603635812E+18</v>
       </c>
       <c r="H14">
-        <v>77657865526.522308</v>
+        <v>10171778682005.789</v>
       </c>
       <c r="I14">
-        <v>-257609934187.74261</v>
+        <v>-33742251593933.82</v>
       </c>
       <c r="J14">
-        <v>618226858.04161501</v>
+        <v>80976559587.817093</v>
       </c>
       <c r="K14">
-        <v>-2.6196029237808518E+17</v>
+        <v>-3.4312069994164031E+19</v>
       </c>
       <c r="L14">
-        <v>44666610930788.688</v>
+        <v>5850519812549753</v>
       </c>
       <c r="M14">
-        <v>-8.33421232053171E+19</v>
+        <v>-1.0916313838724019E+22</v>
       </c>
       <c r="N14">
-        <v>5.1421355123069013E+20</v>
+        <v>6.735269380563232E+22</v>
       </c>
       <c r="O14">
-        <v>-8819214715465.3027</v>
+        <v>-1155157943456021</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1108,46 +1120,46 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>-79438170.225813538</v>
+        <v>-10404966463.62903</v>
       </c>
       <c r="C15">
-        <v>-6696.4673795275576</v>
+        <v>-877116.35742244858</v>
       </c>
       <c r="D15">
-        <v>-65782311.962163098</v>
+        <v>-8616295515.3752079</v>
       </c>
       <c r="E15">
-        <v>-1275313.6268447719</v>
+        <v>-167043066.07526791</v>
       </c>
       <c r="F15">
-        <v>2088542.5451891101</v>
+        <v>273561375.83206213</v>
       </c>
       <c r="G15">
-        <v>-1593910278.2272379</v>
+        <v>-208773476829.13821</v>
       </c>
       <c r="H15">
-        <v>-242910.15354982379</v>
+        <v>-31816845.65714718</v>
       </c>
       <c r="I15">
-        <v>4164.2213266783583</v>
+        <v>545437.83080664929</v>
       </c>
       <c r="J15">
-        <v>105944.69571676719</v>
+        <v>13876842.86784005</v>
       </c>
       <c r="K15">
-        <v>4492759863.6256037</v>
+        <v>588470449121.35229</v>
       </c>
       <c r="L15">
-        <v>-766080.2506618374</v>
+        <v>-100342685.3101752</v>
       </c>
       <c r="M15">
-        <v>1429381826137.4431</v>
+        <v>187223219296257.41</v>
       </c>
       <c r="N15">
-        <v>-8819214715465.3027</v>
+        <v>-1155157943456021</v>
       </c>
       <c r="O15">
-        <v>1114980.2872194371</v>
+        <v>146042292.55466709</v>
       </c>
     </row>
   </sheetData>
@@ -1208,658 +1220,658 @@
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2">
-        <v>5.5188032114100258E-3</v>
-      </c>
-      <c r="C2" s="2">
-        <v>-1.281185083261752</v>
-      </c>
-      <c r="D2" s="2">
-        <v>9.3807993955828013E-3</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1.0957901475150659E-2</v>
-      </c>
-      <c r="F2" s="2">
-        <v>-4.2723903591161829E-4</v>
-      </c>
-      <c r="G2" s="2">
-        <v>-8.3126168452549737E-6</v>
-      </c>
-      <c r="H2" s="2">
-        <v>3.066539244928898E-3</v>
-      </c>
-      <c r="I2" s="2">
-        <v>-4.1070628679678424E-3</v>
-      </c>
-      <c r="J2" s="2">
-        <v>-3.3016625877094511E-4</v>
-      </c>
-      <c r="K2" s="2">
-        <v>2.1848446011543519E-4</v>
-      </c>
-      <c r="L2" s="2">
-        <v>-8.9358106878328999E-2</v>
-      </c>
-      <c r="M2" s="2">
-        <v>1.818993130703116E-8</v>
-      </c>
-      <c r="N2" s="2">
-        <v>3.1443453716340739E-9</v>
-      </c>
-      <c r="O2" s="2">
-        <v>9.0223197967382088E-4</v>
+      <c r="B2">
+        <v>4.2134074192666869E-5</v>
+      </c>
+      <c r="C2">
+        <v>-9.7813865225494651E-3</v>
+      </c>
+      <c r="D2">
+        <v>7.1619023650423952E-5</v>
+      </c>
+      <c r="E2">
+        <v>8.3659629826150211E-5</v>
+      </c>
+      <c r="F2">
+        <v>-3.2618161125742238E-6</v>
+      </c>
+      <c r="G2">
+        <v>-6.3463834725808211E-8</v>
+      </c>
+      <c r="H2">
+        <v>2.341192231558977E-5</v>
+      </c>
+      <c r="I2">
+        <v>-3.1355945295373479E-5</v>
+      </c>
+      <c r="J2">
+        <v>-2.5207004326968918E-6</v>
+      </c>
+      <c r="K2">
+        <v>1.6680501369238931E-6</v>
+      </c>
+      <c r="L2">
+        <v>-6.8221695188254894E-4</v>
+      </c>
+      <c r="M2">
+        <v>1.3887357202108851E-10</v>
+      </c>
+      <c r="N2">
+        <v>2.4005944060822889E-11</v>
+      </c>
+      <c r="O2">
+        <v>6.8882161067056633E-6</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
-        <v>-1.2811852531484409</v>
-      </c>
-      <c r="C3" s="2">
-        <v>3631.2693781444709</v>
-      </c>
-      <c r="D3" s="2">
-        <v>3.7448510958720722</v>
-      </c>
-      <c r="E3" s="2">
-        <v>-15.23403571937329</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0.32131083838190377</v>
-      </c>
-      <c r="G3" s="2">
-        <v>1.077489179536311E-2</v>
-      </c>
-      <c r="H3" s="2">
-        <v>-3.4696011060817802</v>
-      </c>
-      <c r="I3" s="2">
-        <v>-2.0191861280930299</v>
-      </c>
-      <c r="J3" s="2">
-        <v>5.8669402016763433E-2</v>
-      </c>
-      <c r="K3" s="2">
-        <v>3.0547481739632291E-2</v>
-      </c>
-      <c r="L3" s="2">
-        <v>180.7472294434491</v>
-      </c>
-      <c r="M3" s="2">
-        <v>1.2816848260025599E-4</v>
-      </c>
-      <c r="N3" s="2">
-        <v>1.688887217419972E-6</v>
-      </c>
-      <c r="O3" s="2">
-        <v>-1.759378776425188</v>
+      <c r="B3">
+        <v>-9.7813878195731271E-3</v>
+      </c>
+      <c r="C3">
+        <v>27.723433420487499</v>
+      </c>
+      <c r="D3">
+        <v>2.8590588913868929E-2</v>
+      </c>
+      <c r="E3">
+        <v>-0.116306374165825</v>
+      </c>
+      <c r="F3">
+        <v>2.4530924884767192E-3</v>
+      </c>
+      <c r="G3">
+        <v>8.2262416856098555E-5</v>
+      </c>
+      <c r="H3">
+        <v>-2.6489154409486251E-2</v>
+      </c>
+      <c r="I3">
+        <v>-1.5415758611211449E-2</v>
+      </c>
+      <c r="J3">
+        <v>4.4791974685796622E-4</v>
+      </c>
+      <c r="K3">
+        <v>2.3321901736879629E-4</v>
+      </c>
+      <c r="L3">
+        <v>1.37993997679499</v>
+      </c>
+      <c r="M3">
+        <v>9.7852018783271353E-7</v>
+      </c>
+      <c r="N3">
+        <v>1.289404542903404E-8</v>
+      </c>
+      <c r="O3">
+        <v>-1.3432223085186349E-2</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2">
-        <v>9.3807686054412642E-3</v>
-      </c>
-      <c r="C4" s="2">
-        <v>3.744855720776008</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.94674819851131864</v>
-      </c>
-      <c r="E4" s="2">
-        <v>1.420900907360112E-2</v>
-      </c>
-      <c r="F4" s="2">
-        <v>-6.69080574452878E-3</v>
-      </c>
-      <c r="G4" s="2">
-        <v>-3.0462417430269991E-5</v>
-      </c>
-      <c r="H4" s="2">
-        <v>7.5418954986731998E-2</v>
-      </c>
-      <c r="I4" s="2">
-        <v>-0.42710951346205012</v>
-      </c>
-      <c r="J4" s="2">
-        <v>-5.9261211665133824E-3</v>
-      </c>
-      <c r="K4" s="2">
-        <v>1.244898408240578E-2</v>
-      </c>
-      <c r="L4" s="2">
-        <v>-1.5859003806452621</v>
-      </c>
-      <c r="M4" s="2">
-        <v>3.2593814080559211E-6</v>
-      </c>
-      <c r="N4" s="2">
-        <v>-1.419645007756101E-7</v>
-      </c>
-      <c r="O4" s="2">
-        <v>-2.0790920286143199E-3</v>
+      <c r="B4">
+        <v>7.1618788578786463E-5</v>
+      </c>
+      <c r="C4">
+        <v>2.859062422334421E-2</v>
+      </c>
+      <c r="D4">
+        <v>7.2280813991296173E-3</v>
+      </c>
+      <c r="E4">
+        <v>1.0848066502418841E-4</v>
+      </c>
+      <c r="F4">
+        <v>-5.108189128140167E-5</v>
+      </c>
+      <c r="G4">
+        <v>-2.3256958201396989E-7</v>
+      </c>
+      <c r="H4">
+        <v>5.7579654921822824E-4</v>
+      </c>
+      <c r="I4">
+        <v>-3.2608272553364E-3</v>
+      </c>
+      <c r="J4">
+        <v>-4.5243800030480422E-5</v>
+      </c>
+      <c r="K4">
+        <v>9.5043508322051638E-5</v>
+      </c>
+      <c r="L4">
+        <v>-1.2107778034581129E-2</v>
+      </c>
+      <c r="M4">
+        <v>2.4884202753469778E-8</v>
+      </c>
+      <c r="N4">
+        <v>-1.0838478161420469E-9</v>
+      </c>
+      <c r="O4">
+        <v>-1.5873118578663089E-5</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2">
-        <v>1.0957898964815039E-2</v>
-      </c>
-      <c r="C5" s="2">
-        <v>-15.23403620821138</v>
-      </c>
-      <c r="D5" s="2">
-        <v>1.4208869856667489E-2</v>
-      </c>
-      <c r="E5" s="2">
-        <v>1.3997420160393199</v>
-      </c>
-      <c r="F5" s="2">
-        <v>-2.147414670007788E-4</v>
-      </c>
-      <c r="G5" s="2">
-        <v>-8.8436800806519214E-4</v>
-      </c>
-      <c r="H5" s="2">
-        <v>-0.1180731146586307</v>
-      </c>
-      <c r="I5" s="2">
-        <v>5.4960097837528964E-3</v>
-      </c>
-      <c r="J5" s="2">
-        <v>8.1673297739886415E-3</v>
-      </c>
-      <c r="K5" s="2">
-        <v>3.4470869932094121E-4</v>
-      </c>
-      <c r="L5" s="2">
-        <v>-0.83174334819254303</v>
-      </c>
-      <c r="M5" s="2">
-        <v>8.3492132137515258E-7</v>
-      </c>
-      <c r="N5" s="2">
-        <v>1.746329584159736E-7</v>
-      </c>
-      <c r="O5" s="2">
-        <v>0.18867430793771969</v>
+      <c r="B5">
+        <v>8.3659610660642204E-5</v>
+      </c>
+      <c r="C5">
+        <v>-0.11630637789792771</v>
+      </c>
+      <c r="D5">
+        <v>1.0847960215305749E-4</v>
+      </c>
+      <c r="E5">
+        <v>1.0686525990356081E-2</v>
+      </c>
+      <c r="F5">
+        <v>-1.639473733027208E-6</v>
+      </c>
+      <c r="G5">
+        <v>-6.7518311195444061E-6</v>
+      </c>
+      <c r="H5">
+        <v>-9.0144569077956795E-4</v>
+      </c>
+      <c r="I5">
+        <v>4.1960054584570477E-5</v>
+      </c>
+      <c r="J5">
+        <v>6.2354620281032449E-5</v>
+      </c>
+      <c r="K5">
+        <v>2.631726726913937E-6</v>
+      </c>
+      <c r="L5">
+        <v>-6.3500608011438798E-3</v>
+      </c>
+      <c r="M5">
+        <v>6.3743234814259987E-9</v>
+      </c>
+      <c r="N5">
+        <v>1.333259720363105E-9</v>
+      </c>
+      <c r="O5">
+        <v>1.44046036511363E-3</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2">
-        <v>-4.2723891170159657E-4</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.32131078078950992</v>
-      </c>
-      <c r="D6" s="2">
-        <v>-6.6908124811561722E-3</v>
-      </c>
-      <c r="E6" s="2">
-        <v>-2.1474256142793539E-4</v>
-      </c>
-      <c r="F6" s="2">
-        <v>1.645162252369232E-3</v>
-      </c>
-      <c r="G6" s="2">
-        <v>5.8639974208896036E-6</v>
-      </c>
-      <c r="H6" s="2">
-        <v>-2.4537412777005281E-2</v>
-      </c>
-      <c r="I6" s="2">
-        <v>2.666926534053793E-3</v>
-      </c>
-      <c r="J6" s="2">
-        <v>7.2167566292326833E-4</v>
-      </c>
-      <c r="K6" s="2">
-        <v>-9.3447383624270305E-5</v>
-      </c>
-      <c r="L6" s="2">
-        <v>7.8182426738478319E-2</v>
-      </c>
-      <c r="M6" s="2">
-        <v>6.1805278196559732E-8</v>
-      </c>
-      <c r="N6" s="2">
-        <v>9.221371704434601E-9</v>
-      </c>
-      <c r="O6" s="2">
-        <v>3.3805015017764907E-4</v>
+      <c r="B6">
+        <v>-3.2618151642754579E-6</v>
+      </c>
+      <c r="C6">
+        <v>2.4530920487795412E-3</v>
+      </c>
+      <c r="D6">
+        <v>-5.108194271312472E-5</v>
+      </c>
+      <c r="E6">
+        <v>-1.639482088584246E-6</v>
+      </c>
+      <c r="F6">
+        <v>1.256022107419734E-5</v>
+      </c>
+      <c r="G6">
+        <v>4.4769507614721338E-8</v>
+      </c>
+      <c r="H6">
+        <v>-1.8733430615988319E-4</v>
+      </c>
+      <c r="I6">
+        <v>2.0361023241396729E-5</v>
+      </c>
+      <c r="J6">
+        <v>5.5097336795384976E-6</v>
+      </c>
+      <c r="K6">
+        <v>-7.1343710654427261E-7</v>
+      </c>
+      <c r="L6">
+        <v>5.9689466041318599E-4</v>
+      </c>
+      <c r="M6">
+        <v>4.7186103169040655E-10</v>
+      </c>
+      <c r="N6">
+        <v>7.0401850667463467E-11</v>
+      </c>
+      <c r="O6">
+        <v>2.5808911031614989E-6</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="2">
-        <v>-8.3126148794684737E-6</v>
-      </c>
-      <c r="C7" s="2">
-        <v>1.07748919153685E-2</v>
-      </c>
-      <c r="D7" s="2">
-        <v>-3.0462352275897171E-5</v>
-      </c>
-      <c r="E7" s="2">
-        <v>-8.8436801158244243E-4</v>
-      </c>
-      <c r="F7" s="2">
-        <v>5.8639967383968238E-6</v>
-      </c>
-      <c r="G7" s="2">
-        <v>5.7890624311636207E-7</v>
-      </c>
-      <c r="H7" s="2">
-        <v>-1.300337584035887E-5</v>
-      </c>
-      <c r="I7" s="2">
-        <v>5.0143061878698233E-6</v>
-      </c>
-      <c r="J7" s="2">
-        <v>-2.7970423974255189E-6</v>
-      </c>
-      <c r="K7" s="2">
-        <v>-5.1772154209810107E-7</v>
-      </c>
-      <c r="L7" s="2">
-        <v>8.0164739675124823E-4</v>
-      </c>
-      <c r="M7" s="2">
-        <v>-3.0196601853231069E-10</v>
-      </c>
-      <c r="N7" s="2">
-        <v>-7.8366400952054641E-11</v>
-      </c>
-      <c r="O7" s="2">
-        <v>-1.181205734478254E-4</v>
+      <c r="B7">
+        <v>-6.3463819717736528E-8</v>
+      </c>
+      <c r="C7">
+        <v>8.2262417772296459E-5</v>
+      </c>
+      <c r="D7">
+        <v>-2.325690845838073E-7</v>
+      </c>
+      <c r="E7">
+        <v>-6.7518311463973453E-6</v>
+      </c>
+      <c r="F7">
+        <v>4.4769502404134861E-8</v>
+      </c>
+      <c r="G7">
+        <v>4.4197405965904873E-9</v>
+      </c>
+      <c r="H7">
+        <v>-9.9276089656552668E-8</v>
+      </c>
+      <c r="I7">
+        <v>3.8282421179224572E-8</v>
+      </c>
+      <c r="J7">
+        <v>-2.135441097981302E-8</v>
+      </c>
+      <c r="K7">
+        <v>-3.9526174480734926E-9</v>
+      </c>
+      <c r="L7">
+        <v>6.1202890549245703E-6</v>
+      </c>
+      <c r="M7">
+        <v>-2.305401758518932E-12</v>
+      </c>
+      <c r="N7">
+        <v>-5.9829923725121064E-13</v>
+      </c>
+      <c r="O7">
+        <v>-9.0180802153651371E-7</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="2">
-        <v>3.0665384501512962E-3</v>
-      </c>
-      <c r="C8" s="2">
-        <v>-3.4696003052004349</v>
-      </c>
-      <c r="D8" s="2">
-        <v>7.5419070690175782E-2</v>
-      </c>
-      <c r="E8" s="2">
-        <v>-0.118073101907837</v>
-      </c>
-      <c r="F8" s="2">
-        <v>-2.453741306737393E-2</v>
-      </c>
-      <c r="G8" s="2">
-        <v>-1.300338472472989E-5</v>
-      </c>
-      <c r="H8" s="2">
-        <v>0.42572483830988239</v>
-      </c>
-      <c r="I8" s="2">
-        <v>-3.2009155770159017E-2</v>
-      </c>
-      <c r="J8" s="2">
-        <v>-8.4294643436179095E-3</v>
-      </c>
-      <c r="K8" s="2">
-        <v>1.0265433957799719E-3</v>
-      </c>
-      <c r="L8" s="2">
-        <v>-1.022312045336405</v>
-      </c>
-      <c r="M8" s="2">
-        <v>-1.189743370475536E-6</v>
-      </c>
-      <c r="N8" s="2">
-        <v>-1.684259836702912E-7</v>
-      </c>
-      <c r="O8" s="2">
-        <v>-1.254391673624527E-2</v>
+      <c r="B8">
+        <v>2.341191624774912E-5</v>
+      </c>
+      <c r="C8">
+        <v>-2.6489148295045731E-2</v>
+      </c>
+      <c r="D8">
+        <v>5.7579743257233566E-4</v>
+      </c>
+      <c r="E8">
+        <v>-9.0144559343185212E-4</v>
+      </c>
+      <c r="F8">
+        <v>-1.873343083767433E-4</v>
+      </c>
+      <c r="G8">
+        <v>-9.9276157485524535E-8</v>
+      </c>
+      <c r="H8">
+        <v>3.2502557594233819E-3</v>
+      </c>
+      <c r="I8">
+        <v>-2.4437837197676261E-4</v>
+      </c>
+      <c r="J8">
+        <v>-6.4355923277737863E-5</v>
+      </c>
+      <c r="K8">
+        <v>7.8372889814882104E-6</v>
+      </c>
+      <c r="L8">
+        <v>-7.8049841453317371E-3</v>
+      </c>
+      <c r="M8">
+        <v>-9.0832619902462818E-9</v>
+      </c>
+      <c r="N8">
+        <v>-1.285871704442209E-9</v>
+      </c>
+      <c r="O8">
+        <v>-9.5768284931572743E-5</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="2">
-        <v>-4.1070494166155699E-3</v>
-      </c>
-      <c r="C9" s="2">
-        <v>-2.0191883578812142</v>
-      </c>
-      <c r="D9" s="2">
-        <v>-0.42710954971867943</v>
-      </c>
-      <c r="E9" s="2">
-        <v>5.4959461168832763E-3</v>
-      </c>
-      <c r="F9" s="2">
-        <v>2.66692374474121E-3</v>
-      </c>
-      <c r="G9" s="2">
-        <v>5.0143369237931394E-6</v>
-      </c>
-      <c r="H9" s="2">
-        <v>-3.2009106295688199E-2</v>
-      </c>
-      <c r="I9" s="2">
-        <v>0.2225199200101971</v>
-      </c>
-      <c r="J9" s="2">
-        <v>2.541848085790388E-3</v>
-      </c>
-      <c r="K9" s="2">
-        <v>-5.6964138537778106E-3</v>
-      </c>
-      <c r="L9" s="2">
-        <v>0.54996503311139666</v>
-      </c>
-      <c r="M9" s="2">
-        <v>-1.443401580909015E-6</v>
-      </c>
-      <c r="N9" s="2">
-        <v>4.0889503451875409E-8</v>
-      </c>
-      <c r="O9" s="2">
-        <v>1.929035104310978E-3</v>
+      <c r="B9">
+        <v>-3.1355842599145161E-5</v>
+      </c>
+      <c r="C9">
+        <v>-1.5415775634840879E-2</v>
+      </c>
+      <c r="D9">
+        <v>-3.2608275321427032E-3</v>
+      </c>
+      <c r="E9">
+        <v>4.1959568510958968E-5</v>
+      </c>
+      <c r="F9">
+        <v>2.036100194600009E-5</v>
+      </c>
+      <c r="G9">
+        <v>3.8282655836925467E-8</v>
+      </c>
+      <c r="H9">
+        <v>-2.4437799425700262E-4</v>
+      </c>
+      <c r="I9">
+        <v>1.698859419316114E-3</v>
+      </c>
+      <c r="J9">
+        <v>1.940609435244156E-5</v>
+      </c>
+      <c r="K9">
+        <v>-4.349006745719559E-5</v>
+      </c>
+      <c r="L9">
+        <v>4.1987848852047911E-3</v>
+      </c>
+      <c r="M9">
+        <v>-1.101985103837301E-8</v>
+      </c>
+      <c r="N9">
+        <v>3.1217662709565062E-10</v>
+      </c>
+      <c r="O9">
+        <v>1.4727488024442801E-5</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="2">
-        <v>-3.3016616039905061E-4</v>
-      </c>
-      <c r="C10" s="2">
-        <v>5.8669348300832702E-2</v>
-      </c>
-      <c r="D10" s="2">
-        <v>-5.9261278948006596E-3</v>
-      </c>
-      <c r="E10" s="2">
-        <v>8.1673287874783722E-3</v>
-      </c>
-      <c r="F10" s="2">
-        <v>7.2167566842997117E-4</v>
-      </c>
-      <c r="G10" s="2">
-        <v>-2.7970417644675812E-6</v>
-      </c>
-      <c r="H10" s="2">
-        <v>-8.429464147061751E-3</v>
-      </c>
-      <c r="I10" s="2">
-        <v>2.5418509012856911E-3</v>
-      </c>
-      <c r="J10" s="2">
-        <v>6.7174135990971532E-4</v>
-      </c>
-      <c r="K10" s="2">
-        <v>-8.2966331069427384E-5</v>
-      </c>
-      <c r="L10" s="2">
-        <v>6.6170466241225995E-2</v>
-      </c>
-      <c r="M10" s="2">
-        <v>5.7682225962111362E-8</v>
-      </c>
-      <c r="N10" s="2">
-        <v>8.4274307980183631E-9</v>
-      </c>
-      <c r="O10" s="2">
-        <v>1.762220143555311E-3</v>
+      <c r="B10">
+        <v>-2.5206996816629192E-6</v>
+      </c>
+      <c r="C10">
+        <v>4.479193367561879E-4</v>
+      </c>
+      <c r="D10">
+        <v>-4.5243851398529708E-5</v>
+      </c>
+      <c r="E10">
+        <v>6.2354612749381962E-5</v>
+      </c>
+      <c r="F10">
+        <v>5.5097337215801894E-6</v>
+      </c>
+      <c r="G10">
+        <v>-2.1354406147407209E-8</v>
+      </c>
+      <c r="H10">
+        <v>-6.4355921777102404E-5</v>
+      </c>
+      <c r="I10">
+        <v>1.9406115847733831E-5</v>
+      </c>
+      <c r="J10">
+        <v>5.1285032664695374E-6</v>
+      </c>
+      <c r="K10">
+        <v>-6.3341804642450377E-7</v>
+      </c>
+      <c r="L10">
+        <v>5.0518766971197125E-4</v>
+      </c>
+      <c r="M10">
+        <v>4.4038301334263799E-10</v>
+      </c>
+      <c r="N10">
+        <v>6.4340397889735562E-11</v>
+      </c>
+      <c r="O10">
+        <v>1.34539158995309E-5</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="2">
-        <v>2.1848406216614109E-4</v>
-      </c>
-      <c r="C11" s="2">
-        <v>3.054754517637611E-2</v>
-      </c>
-      <c r="D11" s="2">
-        <v>1.2448984742517931E-2</v>
-      </c>
-      <c r="E11" s="2">
-        <v>3.4471055224239241E-4</v>
-      </c>
-      <c r="F11" s="2">
-        <v>-9.3447299242156921E-5</v>
-      </c>
-      <c r="G11" s="2">
-        <v>-5.1772242627792185E-7</v>
-      </c>
-      <c r="H11" s="2">
-        <v>1.026541917811745E-3</v>
-      </c>
-      <c r="I11" s="2">
-        <v>-5.6964136734965866E-3</v>
-      </c>
-      <c r="J11" s="2">
-        <v>-8.2966246241999045E-5</v>
-      </c>
-      <c r="K11" s="2">
-        <v>1.6560834800286009E-4</v>
-      </c>
-      <c r="L11" s="2">
-        <v>-2.219980500410423E-2</v>
-      </c>
-      <c r="M11" s="2">
-        <v>4.2072489752255488E-8</v>
-      </c>
-      <c r="N11" s="2">
-        <v>-1.7469956479837191E-9</v>
-      </c>
-      <c r="O11" s="2">
-        <v>-1.3607755452248901E-5</v>
+      <c r="B11">
+        <v>1.6680470987244071E-6</v>
+      </c>
+      <c r="C11">
+        <v>2.3321950168548019E-4</v>
+      </c>
+      <c r="D11">
+        <v>9.5043513361770104E-5</v>
+      </c>
+      <c r="E11">
+        <v>2.6317408733016429E-6</v>
+      </c>
+      <c r="F11">
+        <v>-7.1343646231723824E-7</v>
+      </c>
+      <c r="G11">
+        <v>-3.9526241984678696E-9</v>
+      </c>
+      <c r="H11">
+        <v>7.8372776977332792E-6</v>
+      </c>
+      <c r="I11">
+        <v>-4.3490066080813407E-5</v>
+      </c>
+      <c r="J11">
+        <v>-6.3341739879765013E-7</v>
+      </c>
+      <c r="K11">
+        <v>1.264360071265292E-6</v>
+      </c>
+      <c r="L11">
+        <v>-1.694875130122067E-4</v>
+      </c>
+      <c r="M11">
+        <v>3.2120830129016999E-10</v>
+      </c>
+      <c r="N11">
+        <v>-1.3337682360956241E-11</v>
+      </c>
+      <c r="O11">
+        <v>-1.038903102461293E-7</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="2">
-        <v>-8.9358088119952106E-2</v>
-      </c>
-      <c r="C12" s="2">
-        <v>180.74722441340961</v>
-      </c>
-      <c r="D12" s="2">
-        <v>-1.585901204450874</v>
-      </c>
-      <c r="E12" s="2">
-        <v>-0.83174349378951085</v>
-      </c>
-      <c r="F12" s="2">
-        <v>7.8182426907306216E-2</v>
-      </c>
-      <c r="G12" s="2">
-        <v>8.0164748831838741E-4</v>
-      </c>
-      <c r="H12" s="2">
-        <v>-1.022312013594515</v>
-      </c>
-      <c r="I12" s="2">
-        <v>0.54996536234758087</v>
-      </c>
-      <c r="J12" s="2">
-        <v>6.6170465511157989E-2</v>
-      </c>
-      <c r="K12" s="2">
-        <v>-2.2199815222992941E-2</v>
-      </c>
-      <c r="L12" s="2">
-        <v>161.79258896349009</v>
-      </c>
-      <c r="M12" s="2">
-        <v>1.085230187175703E-4</v>
-      </c>
-      <c r="N12" s="2">
-        <v>4.7374770315842793E-6</v>
-      </c>
-      <c r="O12" s="2">
-        <v>-6.4286352134673805E-2</v>
+      <c r="B12">
+        <v>-6.8221680866909959E-4</v>
+      </c>
+      <c r="C12">
+        <v>1.37993993839245</v>
+      </c>
+      <c r="D12">
+        <v>-1.210778432404017E-2</v>
+      </c>
+      <c r="E12">
+        <v>-6.3500619127242726E-3</v>
+      </c>
+      <c r="F12">
+        <v>5.9689466170212619E-4</v>
+      </c>
+      <c r="G12">
+        <v>6.1202897540066877E-6</v>
+      </c>
+      <c r="H12">
+        <v>-7.80498390299384E-3</v>
+      </c>
+      <c r="I12">
+        <v>4.1987873988044398E-3</v>
+      </c>
+      <c r="J12">
+        <v>5.0518766413816508E-4</v>
+      </c>
+      <c r="K12">
+        <v>-1.694875910297403E-4</v>
+      </c>
+      <c r="L12">
+        <v>1.2352281257496851</v>
+      </c>
+      <c r="M12">
+        <v>8.2853414899895062E-7</v>
+      </c>
+      <c r="N12">
+        <v>3.6168930307596192E-8</v>
+      </c>
+      <c r="O12">
+        <v>-4.9080313732118193E-4</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="2">
-        <v>1.8189729831986501E-8</v>
-      </c>
-      <c r="C13" s="2">
-        <v>1.2816848016298179E-4</v>
-      </c>
-      <c r="D13" s="2">
-        <v>3.2593756933017469E-6</v>
-      </c>
-      <c r="E13" s="2">
-        <v>8.3492177255701039E-7</v>
-      </c>
-      <c r="F13" s="2">
-        <v>6.1805345425251353E-8</v>
-      </c>
-      <c r="G13" s="2">
-        <v>-3.0196608363349352E-10</v>
-      </c>
-      <c r="H13" s="2">
-        <v>-1.189744278363214E-6</v>
-      </c>
-      <c r="I13" s="2">
-        <v>-1.443398860038581E-6</v>
-      </c>
-      <c r="J13" s="2">
-        <v>5.7682288356528667E-8</v>
-      </c>
-      <c r="K13" s="2">
-        <v>4.2072411611850467E-8</v>
-      </c>
-      <c r="L13" s="2">
-        <v>1.085230265569252E-4</v>
-      </c>
-      <c r="M13" s="2">
-        <v>1.373051010260969E-10</v>
-      </c>
-      <c r="N13" s="2">
-        <v>9.6807204967392587E-12</v>
-      </c>
-      <c r="O13" s="2">
-        <v>9.7616990958306842E-8</v>
+      <c r="B13">
+        <v>1.3887203383171039E-10</v>
+      </c>
+      <c r="C13">
+        <v>9.7852016922500269E-7</v>
+      </c>
+      <c r="D13">
+        <v>2.488415912338058E-8</v>
+      </c>
+      <c r="E13">
+        <v>6.3743269260369314E-9</v>
+      </c>
+      <c r="F13">
+        <v>4.7186154495724584E-10</v>
+      </c>
+      <c r="G13">
+        <v>-2.3054022555430071E-12</v>
+      </c>
+      <c r="H13">
+        <v>-9.0832689216416032E-9</v>
+      </c>
+      <c r="I13">
+        <v>-1.1019830265507531E-8</v>
+      </c>
+      <c r="J13">
+        <v>4.4038348970153469E-10</v>
+      </c>
+      <c r="K13">
+        <v>3.2120770471633028E-10</v>
+      </c>
+      <c r="L13">
+        <v>8.2853420884960093E-7</v>
+      </c>
+      <c r="M13">
+        <v>1.0482749777532101E-12</v>
+      </c>
+      <c r="N13">
+        <v>7.3908813201525527E-14</v>
+      </c>
+      <c r="O13">
+        <v>7.4527055630442396E-10</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="2">
-        <v>3.144338194957824E-9</v>
-      </c>
-      <c r="C14" s="2">
-        <v>1.688883549682678E-6</v>
-      </c>
-      <c r="D14" s="2">
-        <v>-1.4196529183134141E-7</v>
-      </c>
-      <c r="E14" s="2">
-        <v>1.7463292662771131E-7</v>
-      </c>
-      <c r="F14" s="2">
-        <v>9.2213763857018137E-9</v>
-      </c>
-      <c r="G14" s="2">
-        <v>-7.8366366086418304E-11</v>
-      </c>
-      <c r="H14" s="2">
-        <v>-1.684260298315625E-7</v>
-      </c>
-      <c r="I14" s="2">
-        <v>4.0889856158725687E-8</v>
-      </c>
-      <c r="J14" s="2">
-        <v>8.4274348339997317E-9</v>
-      </c>
-      <c r="K14" s="2">
-        <v>-1.7470060217233901E-9</v>
-      </c>
-      <c r="L14" s="2">
-        <v>4.7374775265476999E-6</v>
-      </c>
-      <c r="M14" s="2">
-        <v>9.6807165417076929E-12</v>
-      </c>
-      <c r="N14" s="2">
-        <v>1.295355820006276E-12</v>
-      </c>
-      <c r="O14" s="2">
-        <v>2.1166551513668691E-8</v>
+      <c r="B14">
+        <v>2.4005889269485341E-11</v>
+      </c>
+      <c r="C14">
+        <v>1.289401742718122E-8</v>
+      </c>
+      <c r="D14">
+        <v>-1.083853855567552E-9</v>
+      </c>
+      <c r="E14">
+        <v>1.3332594776711759E-9</v>
+      </c>
+      <c r="F14">
+        <v>7.0401886407252061E-11</v>
+      </c>
+      <c r="G14">
+        <v>-5.9829897106463866E-13</v>
+      </c>
+      <c r="H14">
+        <v>-1.285872056866885E-9</v>
+      </c>
+      <c r="I14">
+        <v>3.1217931988537848E-10</v>
+      </c>
+      <c r="J14">
+        <v>6.4340428702999227E-11</v>
+      </c>
+      <c r="K14">
+        <v>-1.333776156072116E-11</v>
+      </c>
+      <c r="L14">
+        <v>3.6168934086463578E-8</v>
+      </c>
+      <c r="M14">
+        <v>7.3908783006284453E-14</v>
+      </c>
+      <c r="N14">
+        <v>9.8895749921299893E-15</v>
+      </c>
+      <c r="O14">
+        <v>1.6159899487555079E-10</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="2">
-        <v>9.0223178401688741E-4</v>
-      </c>
-      <c r="C15" s="2">
-        <v>-1.759378859458596</v>
-      </c>
-      <c r="D15" s="2">
-        <v>-2.079110383161237E-3</v>
-      </c>
-      <c r="E15" s="2">
-        <v>0.18867430732906479</v>
-      </c>
-      <c r="F15" s="2">
-        <v>3.3805026528097709E-4</v>
-      </c>
-      <c r="G15" s="2">
-        <v>-1.181205726982876E-4</v>
-      </c>
-      <c r="H15" s="2">
-        <v>-1.25439179162168E-2</v>
-      </c>
-      <c r="I15" s="2">
-        <v>1.929043341876873E-3</v>
-      </c>
-      <c r="J15" s="2">
-        <v>1.7622202443680101E-3</v>
-      </c>
-      <c r="K15" s="2">
-        <v>-1.360799685134756E-5</v>
-      </c>
-      <c r="L15" s="2">
-        <v>-6.4286336182824561E-2</v>
-      </c>
-      <c r="M15" s="2">
-        <v>9.7616906825073654E-8</v>
-      </c>
-      <c r="N15" s="2">
-        <v>2.1166552265420331E-8</v>
-      </c>
-      <c r="O15" s="2">
-        <v>2.7399003980134919E-2</v>
+      <c r="B15">
+        <v>6.8882146129354679E-6</v>
+      </c>
+      <c r="C15">
+        <v>-1.3432223719116501E-2</v>
+      </c>
+      <c r="D15">
+        <v>-1.587325870901599E-5</v>
+      </c>
+      <c r="E15">
+        <v>1.440460360466769E-3</v>
+      </c>
+      <c r="F15">
+        <v>2.5808919819339391E-6</v>
+      </c>
+      <c r="G15">
+        <v>-9.0180801581406214E-7</v>
+      </c>
+      <c r="H15">
+        <v>-9.5768293940230197E-5</v>
+      </c>
+      <c r="I15">
+        <v>1.472755091529056E-5</v>
+      </c>
+      <c r="J15">
+        <v>1.3453916669199531E-5</v>
+      </c>
+      <c r="K15">
+        <v>-1.038921532412758E-7</v>
+      </c>
+      <c r="L15">
+        <v>-4.9080301553456002E-4</v>
+      </c>
+      <c r="M15">
+        <v>7.4526991397750032E-10</v>
+      </c>
+      <c r="N15">
+        <v>1.6159900061490369E-10</v>
+      </c>
+      <c r="O15">
+        <v>2.0918152401546279E-4</v>
       </c>
     </row>
   </sheetData>
@@ -1871,6 +1883,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
@@ -1882,7 +1897,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>7.4288647930959309E-2</v>
+        <v>6.4910765049155652E-3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1890,7 +1905,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>60.26001475393506</v>
+        <v>5.2653046844876412</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1898,7 +1913,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.97300986557758939</v>
+        <v>8.5018123945013138E-2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1906,7 +1921,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1.1831069334761419</v>
+        <v>0.1033756547275812</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1914,7 +1929,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>4.0560599753569133E-2</v>
+        <v>3.544040219043421E-3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1922,7 +1937,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>7.6085888515306315E-4</v>
+        <v>6.6481129627816093E-5</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1930,7 +1945,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.65247592929538967</v>
+        <v>5.7011014369360083E-2</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1938,7 +1953,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.47172017129882959</v>
+        <v>4.121722236294089E-2</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1946,7 +1961,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>2.5917973684486121E-2</v>
+        <v>2.264619894478881E-3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1954,7 +1969,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>1.28688907059956E-2</v>
+        <v>1.124437668910683E-3</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -1962,7 +1977,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>12.71977157670255</v>
+        <v>1.1114081724324709</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -1970,7 +1985,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>1.171772593236831E-5</v>
+        <v>1.023853005930641E-6</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -1978,7 +1993,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>1.1381369952717801E-6</v>
+        <v>9.9446342276274737E-8</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -1986,7 +2001,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.16552644495709709</v>
+        <v>1.4463109071546919E-2</v>
       </c>
     </row>
   </sheetData>
@@ -2015,7 +2030,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>8.8049250533327257</v>
+        <v>100.77003049496891</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -2029,13 +2044,13 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.48992750593455509</v>
+        <v>5.6070902834842773</v>
       </c>
       <c r="C3">
-        <v>0.62419870551024426</v>
+        <v>2.1264273897259048E-8</v>
       </c>
       <c r="D3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2043,10 +2058,10 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>5.4365745987815783</v>
+        <v>62.220153469680078</v>
       </c>
       <c r="C4">
-        <v>5.5924432196263751E-8</v>
+        <v>0</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
@@ -2057,10 +2072,10 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>4.1485566567647849</v>
+        <v>47.479129950579072</v>
       </c>
       <c r="C5">
-        <v>3.3805959183341727E-5</v>
+        <v>0</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -2071,7 +2086,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>10.87271842328709</v>
+        <v>124.4353768420938</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -2085,10 +2100,10 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>3.601835243378031</v>
+        <v>41.222048468848271</v>
       </c>
       <c r="C7">
-        <v>3.1790486960026071E-4</v>
+        <v>0</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -2099,7 +2114,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>12.17525510928526</v>
+        <v>139.34256353292989</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -2113,10 +2128,10 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>6.9266541960743098</v>
+        <v>79.273719008240192</v>
       </c>
       <c r="C9">
-        <v>4.6447290458218049E-12</v>
+        <v>0</v>
       </c>
       <c r="D9" t="b">
         <v>1</v>
@@ -2127,7 +2142,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>38.58326318922748</v>
+        <v>441.57520758251292</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -2141,10 +2156,10 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>6.2165420336290582</v>
+        <v>71.14667376583111</v>
       </c>
       <c r="C11">
-        <v>5.3384363596364892E-10</v>
+        <v>0</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
@@ -2155,13 +2170,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>1.6811481194943521</v>
+        <v>19.24029406745295</v>
       </c>
       <c r="C12">
-        <v>9.2773393566236928E-2</v>
+        <v>0</v>
       </c>
       <c r="D12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -2169,13 +2184,13 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>1.1559251877315331</v>
+        <v>13.229257002422729</v>
       </c>
       <c r="C13">
-        <v>0.2477464650218191</v>
+        <v>0</v>
       </c>
       <c r="D13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -2183,13 +2198,13 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>1.9538861441995681</v>
+        <v>22.361708378217521</v>
       </c>
       <c r="C14">
-        <v>5.0749669247421643E-2</v>
+        <v>0</v>
       </c>
       <c r="D14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2197,7 +2212,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>48.108472583574368</v>
+        <v>550.58870120401593</v>
       </c>
       <c r="C15">
         <v>0</v>

</xml_diff>